<commit_message>
Updated excel from current year, updated c43a
</commit_message>
<xml_diff>
--- a/sandbox/analytics_quad_concurrent_course.xlsx
+++ b/sandbox/analytics_quad_concurrent_course.xlsx
@@ -1,26 +1,34 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+<workbook xmlns="http://purl.oclc.org/ooxml/spreadsheetml/main" xmlns:r="http://purl.oclc.org/ooxml/officeDocument/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2" conformance="strict">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10913"/>
-  <workbookPr defaultThemeVersion="202300"/>
+  <workbookPr dateCompatibility="0" defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/muhdkhairulhassan/rrr/utValidateR/data/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/muhdkhairulhassan/rrr/utValidateR/sandbox/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{ECBA025C-BBE9-FB45-806B-C4BB350B2D16}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:9_{96320CE0-60D4-AB4F-AFD4-5AA45AFE22D9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1480" yWindow="880" windowWidth="27240" windowHeight="16440" xr2:uid="{DFD482B2-410E-0348-9688-91753B57A3B7}"/>
+    <workbookView xWindow="0" yWindow="500" windowWidth="35840" windowHeight="20200" xr2:uid="{34ADC7C7-B734-874F-8A25-21993482630C}"/>
   </bookViews>
   <sheets>
-    <sheet name="courses-filtered (1)" sheetId="1" r:id="rId1"/>
+    <sheet name="analytics_quad_concurrent_cours" sheetId="1" r:id="rId1"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">analytics_quad_concurrent_cours!$A$1:$H$121</definedName>
+  </definedNames>
   <calcPr calcId="0"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{79F54976-1DA5-4618-B147-4CDE4B953A38}">
+      <x14:workbookPr/>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="687" uniqueCount="382">
+<sst xmlns="http://purl.oclc.org/ooxml/spreadsheetml/main" count="677" uniqueCount="383">
   <si>
     <t>Utah Tech University</t>
   </si>
@@ -28,19 +36,19 @@
     <t>ACCT</t>
   </si>
   <si>
-    <t>Financial Accounting</t>
+    <t>Principles of Accounting I</t>
   </si>
   <si>
     <t>Accounting II CE</t>
   </si>
   <si>
-    <t>Required of students pursuing majors and emphases in the School of Business, and open to other interested students. Introduces basic concepts of financial accounting, covering complete accounting cycle for service and merchandise companies, including depreciation, accounts receivable, and inventory. Course fee required.</t>
+    <t>Required of students pursuing majors and emphases in the College of Business, and open to other interested students. This course will explain the role of accounting in society and business enabling students to understand career opportunities. Basic concepts of financial and managerial accounting will be taught, while introducing the accounting cycle for service, merchandise, and manufacturing companies. Inclusive Access Course Material (electronic book) fees may apply.</t>
   </si>
   <si>
     <t>ART</t>
   </si>
   <si>
-    <t>FA</t>
+    <t>AR</t>
   </si>
   <si>
     <t>Intro to Art</t>
@@ -118,6 +126,15 @@
     <t>LS</t>
   </si>
   <si>
+    <t>General Biology</t>
+  </si>
+  <si>
+    <t>Biology CE with SEEd</t>
+  </si>
+  <si>
+    <t>Fulfills General Education Life Sciences requirement. Not for science majors, this course focuses on general principles of Biology, including cell theory, genetics, evolution, and interrelationships of living things, using a variety of teaching methods including lecture/discussion, laboratory, overheads, videos, quizzes and exams. Recommended corequisite: BIOL 1015.</t>
+  </si>
+  <si>
     <t>General Biology (lecture only)</t>
   </si>
   <si>
@@ -127,36 +144,27 @@
     <t>Fulfills General Education Life Sciences requirement. Not for science majors, this course focuses on general principles of Biology, including cell theory, genetics, evolution, and interrelationships of living things, using a variety of teaching methods including lecture/discussion, laboratory, overheads, videos, quizzes and exams.</t>
   </si>
   <si>
-    <t>General Biology</t>
-  </si>
-  <si>
-    <t>Biology CE with SEEd</t>
-  </si>
-  <si>
-    <t>Fulfills General Education Life Sciences requirement. Not for science majors, this course focuses on general principles of Biology, including cell theory, genetics, evolution, and interrelationships of living things, using a variety of teaching methods including lecture/discussion, laboratory, overheads, videos, quizzes and exams. Recommended corequisite: BIOL 1015.</t>
+    <t>General Biology Lab</t>
+  </si>
+  <si>
+    <t>Lab course designed recommended but not required to accompany BIOL 1010. Students will have hands-on experience in a laboratory setting, including the use of microscopes, measurement and simple data analysis, observations of osmosis and diffusion, and other group activities in order to appreciate the true essence of science and the scientific process of acquiring knowledge through inquiry. Lab fee required. Corequisite: BIOL 1010.</t>
+  </si>
+  <si>
+    <t>Human Biology</t>
+  </si>
+  <si>
+    <t>Covers basic anatomy and physiology of humans for pre-health science majors. Focuses on the general structure and function of the human body including tissues, organs, and systems. Through lecture, videos, models, quizzes, and tests, students become familiar with how the human body functions. **COURSE LEARNING OUTCOMES (CLOs) At the successful conclusion of this course, students will be able to: 1. Explain the process and methods of science, including asking testable questions, using inductive and deductive reasoning in forming hypotheses and in making reliable predictions. 2. Explain and apply major concepts of life organisms including: the chemistry of life, the cell, the genetic basis of life, and human evolution. 3. Describe the function and processes of the major body systems including: cardiovascular, immune, digestive, urinary, muscular, skeletal, nervous, endocrine, and reproduction, as well as the coordination between systems in maintaining body homeostasis.</t>
+  </si>
+  <si>
+    <t>Principles of Biology I</t>
+  </si>
+  <si>
+    <t>Fulfills General Education Life Sciences requirement. Introductory course required of all Biology majors, including pre-health science, pre-nursing, pre-veterinary, pre-medical, pre-dental, and other pre-professional students. Emphasizes the scientific method; cell processes, including basic chemistry, cellular level structure, and function; and the principles of inheritance, evolution and ecology. Fulfills prerequisite to most other Biology courses. Corequisite: BIOL 1615.</t>
   </si>
   <si>
     <t>LS Lab</t>
   </si>
   <si>
-    <t>General Biology Lab</t>
-  </si>
-  <si>
-    <t>Lab course designed recommended but not required to accompany BIOL 1010. Students will have hands-on experience in a laboratory setting, including the use of microscopes, measurement and simple data analysis, observations of osmosis and diffusion, and other group activities in order to appreciate the true essence of science and the scientific process of acquiring knowledge through inquiry. Lab fee required. Corequisite: BIOL 1010.</t>
-  </si>
-  <si>
-    <t>Human Biology</t>
-  </si>
-  <si>
-    <t>Covers basic anatomy and physiology of humans for pre-health science majors. Focuses on the general structure and function of the human body including tissues, organs, and systems. Through lecture, videos, models, quizzes, and tests, students become familiar with how the human body functions. **COURSE LEARNING OUTCOMES (CLOs) At the successful conclusion of this course, students will be able to: 1. Explain the process and methods of science, including asking testable questions, using inductive and deductive reasoning in forming hypotheses and in making reliable predictions. 2. Explain and apply major concepts of life organisms including: the chemistry of life, the cell, the genetic basis of life, and human evolution. 3. Describe the function and processes of the major body systems including: cardiovascular, immune, digestive, urinary, muscular, skeletal, nervous, endocrine, and reproduction, as well as the coordination between systems in maintaining body homeostasis.</t>
-  </si>
-  <si>
-    <t>Principles of Biology I</t>
-  </si>
-  <si>
-    <t>Fulfills General Education Life Sciences requirement. Introductory course required of all Biology majors, including pre-health science, pre-nursing, pre-veterinary, pre-medical, pre-dental, and other pre-professional students. Emphasizes the scientific method; cell processes, including basic chemistry, cellular level structure, and function; and the principles of inheritance, evolution and ecology. Fulfills prerequisite to most other Biology courses. Corequisite: BIOL 1615.</t>
-  </si>
-  <si>
     <t>Principles of Biology I Lab</t>
   </si>
   <si>
@@ -181,6 +189,15 @@
     <t>PS</t>
   </si>
   <si>
+    <t>Intro to Chemistry</t>
+  </si>
+  <si>
+    <t>Chemistry CE with SEEd</t>
+  </si>
+  <si>
+    <t>Fulfills General Education Physical Science requirement for students majoring in Business, Communication, Fine Arts, Humanities, and other non-Science disciplines. Emphasizes basic chemical concepts within daily life. CHEM 1015 lab course recommended but not required.</t>
+  </si>
+  <si>
     <t>Introduction to Chemistry</t>
   </si>
   <si>
@@ -190,46 +207,32 @@
     <t>Fulfills General Education Physical Science requirement for students majoring in Business, Communication, Fine Arts, Humanities, and other non-Science disciplines. Emphasizes basic chemical concepts within daily life. CHEM 1015 lab course recommended but not required. Inclusive Access Course Material fees may apply, see Fees tab under each course section for details.</t>
   </si>
   <si>
-    <t>Intro to Chemistry</t>
-  </si>
-  <si>
-    <t>Chemistry CE with SEEd</t>
-  </si>
-  <si>
-    <t>Fulfills General Education Physical Science requirement for students majoring in Business, Communication, Fine Arts, Humanities, and other non-Science disciplines. Emphasizes basic chemical concepts within daily life. CHEM 1015 lab course recommended but not required.</t>
+    <t>Intro to Chemistry Lab</t>
+  </si>
+  <si>
+    <t>Lab portion of CHEM 1010. Lab fee required. Corequisite: CHEM 1010.</t>
+  </si>
+  <si>
+    <t>Elementary General/Organic Chemistry</t>
+  </si>
+  <si>
+    <t>Fulfills General Education Physical Science requirement for students majoring in Health Sciences, Family &amp; Consumer Science, Natural Resources, or Agriculture. Not appropriate for students majoring in Life Sciences, Physical Sciences, pre-Medical, pre-Dental or other pre-professional program. First semester in a 2-course sequence covering fundamental laws and reactions of general inorganic and organic chemistry, including the basic organic functional groups. Successful completion satisfies prerequisite for CHEM 1120. Prerequisite: MATH 1000 or MATH 1010 or Math Placement score 23 or higher. Corequisite: CHEM 1115.</t>
   </si>
   <si>
     <t>PS Lab</t>
   </si>
   <si>
-    <t>Intro to Chemistry Lab</t>
-  </si>
-  <si>
-    <t>Lab portion of CHEM 1010. Lab fee required. Corequisite: CHEM 1010.</t>
-  </si>
-  <si>
-    <t>Elementary General/Organic Chemistry</t>
-  </si>
-  <si>
-    <t>Fulfills General Education Physical Science requirement for students majoring in Health Sciences, Family &amp; Consumer Science, Natural Resources, or Agriculture. Not appropriate for students majoring in Life Sciences, Physical Sciences, pre-Medical, pre-Dental or other pre-professional program. First semester in a 2-course sequence covering fundamental laws and reactions of general inorganic and organic chemistry, including the basic organic functional groups. Successful completion satisfies prerequisite for CHEM 1120. Prerequisite: MATH 1000 or MATH 1010 or Math Placement score 23 or higher. Corequisite: CHEM 1115.</t>
-  </si>
-  <si>
     <t>Elementary General/Organic Chemistry Lab</t>
   </si>
   <si>
     <t>Lab portion of CHEM 1110. Successful completion satisfies pre-requisite for CHEM 1125. Lab fee required. Corequisite: CHEM 1110.</t>
   </si>
   <si>
-    <t>Integrated Chemistry for Health Sciences</t>
-  </si>
-  <si>
-    <t>Fulfills the General Education Physical Sciences Requirement and is a course designed to introduce relevant chemistry to students interested in the Health Professions. In particular this will meet the needs of pre-Nursing, Dental Hygiene, and other allied health students to become acquainted with key aspects of chemistry. Key aspects of General/Inorganic, Organic, and Biological Chemistry will be discussed. Four hours of lecture per week. Not appropriate for students majoring in Life Sciences, Physical Sciences, pre-Medical, or pre-Dental programs. Inclusive Access Course Material (electronic book) fees may apply, see Fees tab under each course section for details.</t>
-  </si>
-  <si>
-    <t>Integrated Chemistry for Health Sciences Laboratory</t>
-  </si>
-  <si>
-    <t>Fulfills General Education Lab requirements and is the Lab portion of CHEM 1150. Application of concept in general, organic, and biochemistry to laboratory techniques and experiments.</t>
+    <t>Integrated Chemistry for Health Sciences w/Lab</t>
+  </si>
+  <si>
+    <t>CHEM 1150: (LECTURE):  Fulfills the General Education Physical Sciences Requirement and is a course designed to introduce relevant chemistry to students interested in the Health Professions. In particular this will meet the needs of pre-Nursing, Dental Hygiene, and other allied health students to become acquainted with key aspects of chemistry. Key aspects of General/Inorganic, Organic, and Biological Chemistry will be discussed. Four hours of lecture per week. Not appropriate for students majoring in Life Sciences, Physical Sciences, pre-Medical, or pre-Dental programs. 4 credit hours.
+ CHEM 1155 (LAB): Fulfills General Education Lab requirements and is the Lab portion of CHEM 1150. Application of concept in general, organic, and biochemistry to laboratory techniques and experiments. 1 credit hour.</t>
   </si>
   <si>
     <t>Principles of Chemistry 1</t>
@@ -502,46 +505,16 @@
     <t>Candidates will research and evaluate technology resources for quality, accuracy, and effectiveness. Candidates will apply state and national technology standards as they design, implement, and assess digital learning experiences to engage students and improve learning in K-12 classrooms to enrich professional practice.</t>
   </si>
   <si>
-    <t>EMS</t>
-  </si>
-  <si>
-    <t>Emergency Medical Technician-Intro to Emergency Medical Services</t>
-  </si>
-  <si>
-    <t>Emergency Medical Tech (EMT) CE</t>
-  </si>
-  <si>
-    <t>Open to students who have current CPR certification (American Heart Association-Health Care Provider/American Red Cross-Professional Rescuer). Presents instruction in the theory and practice of first aid, providing students with knowledge and skills necessary to meet common emergencies associated with injury and illness. Topics include CPR, well-being, roles and responsibilities, medical/legal, ethics, lifting &amp; moving, Pt assessment, Airway management, Packaging, bandage/splint, Hazardous Materials, Triage &amp; Terrorism, Mass Casualty Incidents, and disaster management.</t>
-  </si>
-  <si>
-    <t>Emergency Medical Technician Practicum</t>
-  </si>
-  <si>
-    <t>A 12 hour clinical rotation shift is required at a contracted clinical site. Hours can be completed in the Hospital Emergency Department or an Ambulance service. The clinical rotation provides hands-on education with an assigned preceptor in a real life situation.</t>
-  </si>
-  <si>
-    <t>Emergency Medical Technician Patient Management</t>
-  </si>
-  <si>
-    <t>Includes basic knowledge and skills necessary to provide basic patient management and transportation. Topics include Cardiac emergency management, respiratory emergencies, endocrine emergencies, allergies &amp; anaphylaxis, bone and joint injuries, dressings and bandages, sudden illness, and emergency childbirth. Successful completion and recommendation from program coordinator and medical director will provide eligibility for testing and certification at the National Registry of Emergency Medical Technician (NREMT) EMT level. Upon successful completion of the NREMT certification, students are eligible for licensure from the Utah Bureau of Emergency Medical Services at the EMT level.</t>
-  </si>
-  <si>
-    <t>Emergency Medical Technician Lab</t>
-  </si>
-  <si>
-    <t>Emergency Medical Technician lab will provide practical learn of skills and National Registry competencies. These competencies include patient assessment, patient history taking, basic airway adjuncts, airway management, insertion of Nasopharyngeal Airway/Orophyryngeal airway (NPA/OPA), basic vital signs, patient assisted medications, suctioning, bandaging, splinting, lifting and moving patients, extraction of patients from cars, home, office, and other various locations. Students are required to complete an 8 station practical exam. Upon successful completion, students may be recommended for testing and licensure at the Emergency Medical Technician (EMT) level.</t>
-  </si>
-  <si>
     <t>ENGL</t>
   </si>
   <si>
-    <t>C</t>
+    <t>WC</t>
   </si>
   <si>
     <t>Intro to Writing</t>
   </si>
   <si>
-    <t>Language Arts 11 or 12 CE (ENG1010)</t>
+    <t>Language Arts 12 CE (ENG1010)</t>
   </si>
   <si>
     <t>Partially fulfills General Education English requirement. Designed to improve students' abilities to read, analyze, and write expository papers. Provides opportunities to write and revise a number of essays. Activities, library research, portfolios, writing to a style guide, and tests may also be used to prepare students to write college level papers. Successful completers (grade C or higher) will be prepared to take ENGL 2010 or ENGL 2010A. Prerequisites: Writing ACT/English placement score of 19; or ENGL 0990 (Grade C or higher); OR ESL 2700 OR ESL 2750 (Grade B or higher); AND ACT/Reading placement score 17 or higher, or ENGL 1470 (Grade C or higher-can be concurrently enrolled); AND LIB 1010 (can be concurrently enrolled); OR LIB 1000.</t>
@@ -658,6 +631,16 @@
     <t>Fulfills the General Education American Institutions (Utah State Code R470) requirement. Surveys the historical, constitutional, and economic growth of the United States from colonial times to the present. Employs lectures, discussion, audio-visual materials, and various other instructional methods. Successful students will demonstrate a reasonable understanding of the history, principles, form of government, and economic system of the United States, as well as an appreciation of the American heritage and the responsibilities of American citizens. Prerequisite: Reading placement score 17 or higher, or ENGL 1470.</t>
   </si>
   <si>
+    <t>American History (Year-Long)</t>
+  </si>
+  <si>
+    <t>U.S. History II CE</t>
+  </si>
+  <si>
+    <t>Fulfills the General Education American Institutions (Utah State Code R470) requirement. Surveys the historical, constitutional, and economic growth of the United States from colonial times to the present. Employs lectures, discussion, audio-visual materials, and various other instructional methods. Successful students will demonstrate a reasonable understanding of the history, principles, form of government, economic system of the United States, and the responsibilities of American citizens.
+ Utah Tech is looking to get this course approved for</t>
+  </si>
+  <si>
     <t>U.S. History to 1877</t>
   </si>
   <si>
@@ -667,9 +650,6 @@
     <t>U.S. History Since 1877</t>
   </si>
   <si>
-    <t>U.S. History II CE</t>
-  </si>
-  <si>
     <t>If both HIST 2700 and HIST 2710 are successfully completed, fulfills the General Education American Institutions (Utah State Code R470) requirement. If course is not used for American Institutions requirement, it can be used to fulfill the General Education Social &amp; Behavioral Sciences requirement.Chronological survey of the second half of the American experience, beginning with the collapse of post-Civil War Reconstruction and emphasizing the growth of the U.S., emergence as a world power, and domestic reform of the twentieth century, through contemporary issues. Includes the social, political, economic, cultural, and diplomatic developments throughout this period. Prerequisite: Reading placement score 17 or higher, or ENGL 1470.</t>
   </si>
   <si>
@@ -718,7 +698,7 @@
     <t>Linux Fundamentals CE</t>
   </si>
   <si>
-    <t>Required of all Computer and Information Technology majors, and open to students with a general interest in computer operating systems. Introduces operating system concepts, including file systems, process management, user management, and security. Students will install and configure LINUX and MAC OSX. Course fee required.</t>
+    <t>Required of all Computer and Information Technology majors, and open to students with a general interest in computer operating systems. Introduces operating system concepts, including file systems, process management, user management, and security. Students will install and configure LINUX and MAC OSX. Introduces operating system concepts, including file systems, process management, user management, and security. Students will install and configure Linux based systems. This course is required of all Information Technology majors, and open to students with a general interest in computer operating systems.</t>
   </si>
   <si>
     <t>A+ Computer Hardware/Windows OS</t>
@@ -748,6 +728,15 @@
     <t>Required of all Computer Science and Computer and Information Technology majors, and open to students with a general interest in computer networking. Introduces fundamental concepts of computer networks, including physical, transport, and application layers through completion of assignments predicting and measuring the behavior of computer networks under various conditions. Course fee required. Prerequisite: IT 1100 (Grade C- or higher).</t>
   </si>
   <si>
+    <t>Information Security</t>
+  </si>
+  <si>
+    <t>Principles of Cyber Defense &amp; Ethics CE</t>
+  </si>
+  <si>
+    <t>Required of students pursuing an Information Technology emphasis. Reviews current security exploits, vulnerabilities, and counter measures. Covers general security models and architectures, encryption and forensics.</t>
+  </si>
+  <si>
     <t>IXD</t>
   </si>
   <si>
@@ -862,24 +851,6 @@
     <t>Fulfills General Education Mathematics requirement. Continuation of MATH 1220. Includes partial derivatives, gradient vectors, Lagrange multipliers, multiple integrals, line integrals, Green's Theorem, surface integrals, the Divergence Theorem, Stokes' Theorem. Required for Utah Level 3 and Level 4 Endorsement. Prerequisite: MATH 1220 (Grade C or higher).</t>
   </si>
   <si>
-    <t>MDIA</t>
-  </si>
-  <si>
-    <t>Introduction to Video Production</t>
-  </si>
-  <si>
-    <t>Television Broadcasting 2 CE</t>
-  </si>
-  <si>
-    <t>For Media Studies majors, but open to all students interested in television production. Covers basic tools of television studio production and processes involved in creating a television program, including basic terminology and the duties of studio production technical positions. Corequisite: MDIA 1385.</t>
-  </si>
-  <si>
-    <t>Introduction to Video Production Lab</t>
-  </si>
-  <si>
-    <t>Lab portion of MDIA 1380 (requires 6 lab hours per week). Lab fee required. Corequisite: MDIA 1380.</t>
-  </si>
-  <si>
     <t>MECH</t>
   </si>
   <si>
@@ -898,6 +869,15 @@
     <t>Lab portion of MECH 1000</t>
   </si>
   <si>
+    <t>Manufacturing Processes</t>
+  </si>
+  <si>
+    <t>Manufacturing Principles 1 CE</t>
+  </si>
+  <si>
+    <t>An introduction to manufacturing processes required for Mechanical Engineering majors and open to makers. Students learn about various manufacturing processes through lecture and tours of local manufacturing facilities. Topics include: advantages and limitations of common manufacturing methods, component assembly, quality control, and manufacturing economics.</t>
+  </si>
+  <si>
     <t>MGMT</t>
   </si>
   <si>
@@ -925,8 +905,7 @@
     <t>Seminar in Entrepreneurship</t>
   </si>
   <si>
-    <t>This seminar course focuses start-up businesses and the management skills needed from inception to business organization. This course draws on the real-life experience of entrepreneurs coupled with a healthy dose of theory in the field of entrepreneurship. It is intended to be cross-disciplined and inclusive of all academic backgrounds at any level. Requirements of this course will include weekly reports on speakers and topics, discussion and participation in class, and attendance in a weekly class. After taking this class, a student will be introduced to the challenges of starting a business, and have experience the process of vetting and validating a business idea.
- This class will be taken as a corequisite with MGMT 2600.</t>
+    <t>This seminar course focuses start-up businesses and the management skills needed from inception to business organization. This course draws on the real-life experience of entrepreneurs coupled with a healthy dose of theory in the field of entrepreneurship. It is intended to be cross-disciplined and inclusive of all academic backgrounds at any level. Requirements of this course will include weekly reports on speakers and topics, discussion and participation in class, and attendance in a weekly class. After taking this class, a student will be introduced to the challenges of starting a business, and have experience the process of vetting and validating a business idea.</t>
   </si>
   <si>
     <t>MUSC</t>
@@ -1026,6 +1005,36 @@
   </si>
   <si>
     <t>Fulfills the General Education American Institutions (Utah State Code R470) requirement. Surveys the founding of the U.S. Government; the U.S. Constitution; and the Legislative, Executive, and Judicial branches of government. Also covers politics and elections, international relations, and national security. Helps students acquire a greater understanding of the federal system and of federalism. Employs a wide variety of instructional methods including lectures, student reports, discussions, and audio-visual materials. Successful students will demonstrate a reasonable understanding of the history, principles, form of government, and economic system of the United States. Prerequisite: Reading placement score 17 or higher, or ENGL 1470.</t>
+  </si>
+  <si>
+    <t>PORT</t>
+  </si>
+  <si>
+    <t>Navigating Identities of the Portuguese-speaking World</t>
+  </si>
+  <si>
+    <t>Portuguese CE 3116</t>
+  </si>
+  <si>
+    <t>In this course students investigate the themes of travel, navigation, and cross-cultural encounters throughout today‚Äôs Portuguese-speaking world.</t>
+  </si>
+  <si>
+    <t>Cultural Issues Through Literature and Film</t>
+  </si>
+  <si>
+    <t>Portuguese CE 3117</t>
+  </si>
+  <si>
+    <t>Analyze and interpret works of literature and film in the Portuguese-speaking world to explore cultural issues.</t>
+  </si>
+  <si>
+    <t>Popular Culture</t>
+  </si>
+  <si>
+    <t>Portuguese CE 3118</t>
+  </si>
+  <si>
+    <t>This course explores ways that popular media and entertainment reflect and shape how Portuguese speakers view themselves, their community, and their own and other cultures. Students will be introduced to the historical contexts and perspectives of popular media as cultural products and practices.</t>
   </si>
   <si>
     <t>PSY</t>
@@ -1168,12 +1177,16 @@
   </si>
   <si>
     <t>Reason</t>
+  </si>
+  <si>
+    <t>CHEM 1150: (LECTURE):  Fulfills the General Education Physical Sciences Requirement and is a course designed to introduce relevant chemistry to students interested in the Health Professions. In particular this will meet the needs of pre-Nursing, Dental Hygiene, and other allied health students to become acquainted with key aspects of chemistry. Key aspects of General/Inorganic, Organic, and Biological Chemistry will be discussed. Four hours of lecture per week. Not appropriate for students majoring in Life Sciences, Physical Sciences, pre-Medical, or pre-Dental programs. 4 credit hours.
+ CHEM 1155 (LAB): Fulfills General Education Lab requirements and is the Lab portion of CHEM 1155. Application of concept in general, organic, and biochemistry to laboratory techniques and experiments. 1 credit hour.</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+<styleSheet xmlns="http://purl.oclc.org/ooxml/spreadsheetml/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="18" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
@@ -1493,15 +1506,15 @@
   </fills>
   <borders count="10">
     <border>
-      <left/>
-      <right/>
+      <start/>
+      <end/>
       <top/>
       <bottom/>
       <diagonal/>
     </border>
     <border>
-      <left/>
-      <right/>
+      <start/>
+      <end/>
       <top/>
       <bottom style="thick">
         <color theme="4"/>
@@ -1509,8 +1522,8 @@
       <diagonal/>
     </border>
     <border>
-      <left/>
-      <right/>
+      <start/>
+      <end/>
       <top/>
       <bottom style="thick">
         <color theme="4" tint="0.499984740745262"/>
@@ -1518,8 +1531,8 @@
       <diagonal/>
     </border>
     <border>
-      <left/>
-      <right/>
+      <start/>
+      <end/>
       <top/>
       <bottom style="medium">
         <color theme="4" tint="0.39997558519241921"/>
@@ -1527,12 +1540,12 @@
       <diagonal/>
     </border>
     <border>
-      <left style="thin">
+      <start style="thin">
         <color rgb="FF7F7F7F"/>
-      </left>
-      <right style="thin">
+      </start>
+      <end style="thin">
         <color rgb="FF7F7F7F"/>
-      </right>
+      </end>
       <top style="thin">
         <color rgb="FF7F7F7F"/>
       </top>
@@ -1542,12 +1555,12 @@
       <diagonal/>
     </border>
     <border>
-      <left style="thin">
+      <start style="thin">
         <color rgb="FF3F3F3F"/>
-      </left>
-      <right style="thin">
+      </start>
+      <end style="thin">
         <color rgb="FF3F3F3F"/>
-      </right>
+      </end>
       <top style="thin">
         <color rgb="FF3F3F3F"/>
       </top>
@@ -1557,8 +1570,8 @@
       <diagonal/>
     </border>
     <border>
-      <left/>
-      <right/>
+      <start/>
+      <end/>
       <top/>
       <bottom style="double">
         <color rgb="FFFF8001"/>
@@ -1566,12 +1579,12 @@
       <diagonal/>
     </border>
     <border>
-      <left style="double">
+      <start style="double">
         <color rgb="FF3F3F3F"/>
-      </left>
-      <right style="double">
+      </start>
+      <end style="double">
         <color rgb="FF3F3F3F"/>
-      </right>
+      </end>
       <top style="double">
         <color rgb="FF3F3F3F"/>
       </top>
@@ -1581,12 +1594,12 @@
       <diagonal/>
     </border>
     <border>
-      <left style="thin">
+      <start style="thin">
         <color rgb="FFB2B2B2"/>
-      </left>
-      <right style="thin">
+      </start>
+      <end style="thin">
         <color rgb="FFB2B2B2"/>
-      </right>
+      </end>
       <top style="thin">
         <color rgb="FFB2B2B2"/>
       </top>
@@ -1596,8 +1609,8 @@
       <diagonal/>
     </border>
     <border>
-      <left/>
-      <right/>
+      <start/>
+      <end/>
       <top style="thin">
         <color theme="4"/>
       </top>
@@ -1715,7 +1728,7 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://purl.oclc.org/ooxml/drawingml/main" name="Office Theme">
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
@@ -1868,25 +1881,25 @@
         </a:solidFill>
         <a:gradFill rotWithShape="1">
           <a:gsLst>
-            <a:gs pos="0">
+            <a:gs pos="0%">
               <a:schemeClr val="phClr">
-                <a:lumMod val="110000"/>
-                <a:satMod val="105000"/>
-                <a:tint val="67000"/>
+                <a:lumMod val="110%"/>
+                <a:satMod val="105%"/>
+                <a:tint val="67%"/>
               </a:schemeClr>
             </a:gs>
-            <a:gs pos="50000">
+            <a:gs pos="50%">
               <a:schemeClr val="phClr">
-                <a:lumMod val="105000"/>
-                <a:satMod val="103000"/>
-                <a:tint val="73000"/>
+                <a:lumMod val="105%"/>
+                <a:satMod val="103%"/>
+                <a:tint val="73%"/>
               </a:schemeClr>
             </a:gs>
-            <a:gs pos="100000">
+            <a:gs pos="100%">
               <a:schemeClr val="phClr">
-                <a:lumMod val="105000"/>
-                <a:satMod val="109000"/>
-                <a:tint val="81000"/>
+                <a:lumMod val="105%"/>
+                <a:satMod val="109%"/>
+                <a:tint val="81%"/>
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
@@ -1894,25 +1907,25 @@
         </a:gradFill>
         <a:gradFill rotWithShape="1">
           <a:gsLst>
-            <a:gs pos="0">
+            <a:gs pos="0%">
               <a:schemeClr val="phClr">
-                <a:satMod val="103000"/>
-                <a:lumMod val="102000"/>
-                <a:tint val="94000"/>
+                <a:satMod val="103%"/>
+                <a:lumMod val="102%"/>
+                <a:tint val="94%"/>
               </a:schemeClr>
             </a:gs>
-            <a:gs pos="50000">
+            <a:gs pos="50%">
               <a:schemeClr val="phClr">
-                <a:satMod val="110000"/>
-                <a:lumMod val="100000"/>
-                <a:shade val="100000"/>
+                <a:satMod val="110%"/>
+                <a:lumMod val="100%"/>
+                <a:shade val="100%"/>
               </a:schemeClr>
             </a:gs>
-            <a:gs pos="100000">
+            <a:gs pos="100%">
               <a:schemeClr val="phClr">
-                <a:lumMod val="99000"/>
-                <a:satMod val="120000"/>
-                <a:shade val="78000"/>
+                <a:lumMod val="99%"/>
+                <a:satMod val="120%"/>
+                <a:shade val="78%"/>
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
@@ -1925,21 +1938,21 @@
             <a:schemeClr val="phClr"/>
           </a:solidFill>
           <a:prstDash val="solid"/>
-          <a:miter lim="800000"/>
+          <a:miter lim="800%"/>
         </a:ln>
         <a:ln w="19050" cap="flat" cmpd="sng" algn="ctr">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
           <a:prstDash val="solid"/>
-          <a:miter lim="800000"/>
+          <a:miter lim="800%"/>
         </a:ln>
         <a:ln w="25400" cap="flat" cmpd="sng" algn="ctr">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
           <a:prstDash val="solid"/>
-          <a:miter lim="800000"/>
+          <a:miter lim="800%"/>
         </a:ln>
       </a:lnStyleLst>
       <a:effectStyleLst>
@@ -1953,7 +1966,7 @@
           <a:effectLst>
             <a:outerShdw blurRad="57150" dist="19050" dir="5400000" algn="ctr" rotWithShape="0">
               <a:srgbClr val="000000">
-                <a:alpha val="63000"/>
+                <a:alpha val="63%"/>
               </a:srgbClr>
             </a:outerShdw>
           </a:effectLst>
@@ -1965,32 +1978,32 @@
         </a:solidFill>
         <a:solidFill>
           <a:schemeClr val="phClr">
-            <a:tint val="95000"/>
-            <a:satMod val="170000"/>
+            <a:tint val="95%"/>
+            <a:satMod val="170%"/>
           </a:schemeClr>
         </a:solidFill>
         <a:gradFill rotWithShape="1">
           <a:gsLst>
-            <a:gs pos="0">
+            <a:gs pos="0%">
               <a:schemeClr val="phClr">
-                <a:tint val="93000"/>
-                <a:satMod val="150000"/>
-                <a:shade val="98000"/>
-                <a:lumMod val="102000"/>
+                <a:tint val="93%"/>
+                <a:satMod val="150%"/>
+                <a:shade val="98%"/>
+                <a:lumMod val="102%"/>
               </a:schemeClr>
             </a:gs>
-            <a:gs pos="50000">
+            <a:gs pos="50%">
               <a:schemeClr val="phClr">
-                <a:tint val="98000"/>
-                <a:satMod val="130000"/>
-                <a:shade val="90000"/>
-                <a:lumMod val="103000"/>
+                <a:tint val="98%"/>
+                <a:satMod val="130%"/>
+                <a:shade val="90%"/>
+                <a:lumMod val="103%"/>
               </a:schemeClr>
             </a:gs>
-            <a:gs pos="100000">
+            <a:gs pos="100%">
               <a:schemeClr val="phClr">
-                <a:shade val="63000"/>
-                <a:satMod val="120000"/>
+                <a:shade val="63%"/>
+                <a:satMod val="120%"/>
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
@@ -2030,9 +2043,14 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E7072C93-06CD-6E46-B6FE-9C96D9C1C7EF}">
+<worksheet xmlns="http://purl.oclc.org/ooxml/spreadsheetml/main" xmlns:r="http://purl.oclc.org/ooxml/officeDocument/relationships" xmlns:v="urn:schemas-microsoft-com:vml" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F61A08E9-A0F5-9448-A2BC-A228F6060EDB}">
+  <sheetPr filterMode="1"/>
   <dimension ref="A1:H121"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="5" max="5" width="60.1640625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="34" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
@@ -2060,7 +2078,7 @@
         <v>381</v>
       </c>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>0</v>
       </c>
@@ -2083,7 +2101,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>0</v>
       </c>
@@ -2109,7 +2127,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>0</v>
       </c>
@@ -2135,7 +2153,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>0</v>
       </c>
@@ -2161,7 +2179,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>0</v>
       </c>
@@ -2187,7 +2205,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>0</v>
       </c>
@@ -2213,7 +2231,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
         <v>0</v>
       </c>
@@ -2239,7 +2257,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
         <v>0</v>
       </c>
@@ -2265,7 +2283,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
         <v>0</v>
       </c>
@@ -2282,7 +2300,7 @@
         <v>32</v>
       </c>
       <c r="F10">
-        <v>8020013012</v>
+        <v>8020013010</v>
       </c>
       <c r="G10" t="s">
         <v>33</v>
@@ -2291,7 +2309,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
         <v>0</v>
       </c>
@@ -2308,7 +2326,7 @@
         <v>35</v>
       </c>
       <c r="F11">
-        <v>8020013010</v>
+        <v>8020013012</v>
       </c>
       <c r="G11" t="s">
         <v>36</v>
@@ -2317,7 +2335,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
         <v>0</v>
       </c>
@@ -2327,23 +2345,20 @@
       <c r="C12">
         <v>1015</v>
       </c>
-      <c r="D12" t="s">
+      <c r="E12" t="s">
         <v>38</v>
-      </c>
-      <c r="E12" t="s">
-        <v>39</v>
       </c>
       <c r="F12">
         <v>8020013010</v>
       </c>
       <c r="G12" t="s">
-        <v>36</v>
+        <v>33</v>
       </c>
       <c r="H12" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.2">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
         <v>0</v>
       </c>
@@ -2357,19 +2372,19 @@
         <v>31</v>
       </c>
       <c r="E13" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="F13">
         <v>8020013010</v>
       </c>
       <c r="G13" t="s">
-        <v>36</v>
+        <v>33</v>
       </c>
       <c r="H13" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="14" spans="1:8" x14ac:dyDescent="0.2">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
         <v>0</v>
       </c>
@@ -2383,19 +2398,19 @@
         <v>31</v>
       </c>
       <c r="E14" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="F14">
         <v>8020013010</v>
       </c>
       <c r="G14" t="s">
-        <v>36</v>
+        <v>33</v>
       </c>
       <c r="H14" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="15" spans="1:8" x14ac:dyDescent="0.2">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="15" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
         <v>0</v>
       </c>
@@ -2406,7 +2421,7 @@
         <v>1615</v>
       </c>
       <c r="D15" t="s">
-        <v>38</v>
+        <v>44</v>
       </c>
       <c r="E15" t="s">
         <v>45</v>
@@ -2415,13 +2430,13 @@
         <v>8020013010</v>
       </c>
       <c r="G15" t="s">
-        <v>36</v>
+        <v>33</v>
       </c>
       <c r="H15" t="s">
         <v>46</v>
       </c>
     </row>
-    <row r="16" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
         <v>0</v>
       </c>
@@ -2461,7 +2476,7 @@
         <v>53</v>
       </c>
       <c r="F17">
-        <v>8030013010</v>
+        <v>8030013012</v>
       </c>
       <c r="G17" t="s">
         <v>54</v>
@@ -2487,7 +2502,7 @@
         <v>56</v>
       </c>
       <c r="F18">
-        <v>8030013012</v>
+        <v>8030013010</v>
       </c>
       <c r="G18" t="s">
         <v>57</v>
@@ -2506,20 +2521,17 @@
       <c r="C19">
         <v>1015</v>
       </c>
-      <c r="D19" t="s">
+      <c r="E19" t="s">
         <v>59</v>
-      </c>
-      <c r="E19" t="s">
-        <v>60</v>
       </c>
       <c r="F19">
         <v>8030013012</v>
       </c>
       <c r="G19" t="s">
-        <v>57</v>
+        <v>54</v>
       </c>
       <c r="H19" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
     </row>
     <row r="20" spans="1:8" x14ac:dyDescent="0.2">
@@ -2536,16 +2548,16 @@
         <v>52</v>
       </c>
       <c r="E20" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="F20">
         <v>8030013012</v>
       </c>
       <c r="G20" t="s">
-        <v>57</v>
+        <v>54</v>
       </c>
       <c r="H20" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
     </row>
     <row r="21" spans="1:8" x14ac:dyDescent="0.2">
@@ -2559,7 +2571,7 @@
         <v>1115</v>
       </c>
       <c r="D21" t="s">
-        <v>59</v>
+        <v>63</v>
       </c>
       <c r="E21" t="s">
         <v>64</v>
@@ -2568,13 +2580,13 @@
         <v>8030013012</v>
       </c>
       <c r="G21" t="s">
-        <v>57</v>
+        <v>54</v>
       </c>
       <c r="H21" t="s">
         <v>65</v>
       </c>
     </row>
-    <row r="22" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:8" ht="409.6" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
         <v>0</v>
       </c>
@@ -2594,13 +2606,13 @@
         <v>8030013012</v>
       </c>
       <c r="G22" t="s">
-        <v>57</v>
-      </c>
-      <c r="H22" t="s">
+        <v>54</v>
+      </c>
+      <c r="H22" s="1" t="s">
         <v>67</v>
       </c>
     </row>
-    <row r="23" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:8" ht="409.6" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
         <v>0</v>
       </c>
@@ -2611,19 +2623,19 @@
         <v>1155</v>
       </c>
       <c r="D23" t="s">
-        <v>59</v>
+        <v>52</v>
       </c>
       <c r="E23" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="F23">
         <v>8030013012</v>
       </c>
       <c r="G23" t="s">
-        <v>57</v>
-      </c>
-      <c r="H23" t="s">
-        <v>69</v>
+        <v>54</v>
+      </c>
+      <c r="H23" s="1" t="s">
+        <v>382</v>
       </c>
     </row>
     <row r="24" spans="1:8" x14ac:dyDescent="0.2">
@@ -2640,16 +2652,16 @@
         <v>52</v>
       </c>
       <c r="E24" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="F24">
         <v>8030013012</v>
       </c>
       <c r="G24" t="s">
-        <v>57</v>
+        <v>54</v>
       </c>
       <c r="H24" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
     </row>
     <row r="25" spans="1:8" x14ac:dyDescent="0.2">
@@ -2663,27 +2675,27 @@
         <v>1215</v>
       </c>
       <c r="D25" t="s">
-        <v>59</v>
+        <v>63</v>
       </c>
       <c r="E25" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="F25">
         <v>8030013012</v>
       </c>
       <c r="G25" t="s">
-        <v>57</v>
+        <v>54</v>
       </c>
       <c r="H25" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="26" spans="1:8" x14ac:dyDescent="0.2">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="26" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
         <v>0</v>
       </c>
       <c r="B26" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="C26">
         <v>1010</v>
@@ -2692,24 +2704,24 @@
         <v>17</v>
       </c>
       <c r="E26" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="F26">
         <v>3020013062</v>
       </c>
       <c r="G26" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="H26" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="27" spans="1:8" x14ac:dyDescent="0.2">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="27" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
       <c r="A27" t="s">
         <v>0</v>
       </c>
       <c r="B27" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="C27">
         <v>1020</v>
@@ -2718,24 +2730,24 @@
         <v>17</v>
       </c>
       <c r="E27" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="F27">
         <v>3020013063</v>
       </c>
       <c r="G27" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="H27" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="28" spans="1:8" x14ac:dyDescent="0.2">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="28" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
       <c r="A28" t="s">
         <v>0</v>
       </c>
       <c r="B28" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="C28">
         <v>2010</v>
@@ -2744,24 +2756,24 @@
         <v>17</v>
       </c>
       <c r="E28" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="F28">
         <v>3020013064</v>
       </c>
       <c r="G28" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="H28" t="s">
-        <v>83</v>
-      </c>
-    </row>
-    <row r="29" spans="1:8" x14ac:dyDescent="0.2">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="29" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
       <c r="A29" t="s">
         <v>0</v>
       </c>
       <c r="B29" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="C29">
         <v>2020</v>
@@ -2770,246 +2782,237 @@
         <v>17</v>
       </c>
       <c r="E29" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="F29">
         <v>3020013068</v>
       </c>
       <c r="G29" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="H29" t="s">
-        <v>86</v>
-      </c>
-    </row>
-    <row r="30" spans="1:8" x14ac:dyDescent="0.2">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="30" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
       <c r="A30" t="s">
         <v>0</v>
       </c>
       <c r="B30" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="C30">
         <v>3116</v>
       </c>
-      <c r="D30" t="s">
-        <v>17</v>
-      </c>
       <c r="E30" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="F30">
         <v>3020013066</v>
       </c>
       <c r="G30" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="H30" t="s">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="31" spans="1:8" x14ac:dyDescent="0.2">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="31" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
       <c r="A31" t="s">
         <v>0</v>
       </c>
       <c r="B31" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="C31">
         <v>3117</v>
       </c>
-      <c r="D31" t="s">
-        <v>17</v>
-      </c>
       <c r="E31" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="F31">
         <v>3020013067</v>
       </c>
       <c r="G31" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="H31" t="s">
-        <v>92</v>
-      </c>
-    </row>
-    <row r="32" spans="1:8" x14ac:dyDescent="0.2">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="32" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
       <c r="A32" t="s">
         <v>0</v>
       </c>
       <c r="B32" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="C32">
         <v>3118</v>
       </c>
-      <c r="D32" t="s">
-        <v>17</v>
-      </c>
       <c r="E32" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="F32">
         <v>3020013065</v>
       </c>
       <c r="G32" t="s">
+        <v>92</v>
+      </c>
+      <c r="H32" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="33" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A33" t="s">
+        <v>0</v>
+      </c>
+      <c r="B33" t="s">
         <v>94</v>
-      </c>
-      <c r="H32" t="s">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="33" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A33" t="s">
-        <v>0</v>
-      </c>
-      <c r="B33" t="s">
-        <v>96</v>
       </c>
       <c r="C33">
         <v>1200</v>
       </c>
       <c r="E33" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="F33">
         <v>32020013216</v>
       </c>
       <c r="G33" t="s">
+        <v>96</v>
+      </c>
+      <c r="H33" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="34" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A34" t="s">
+        <v>0</v>
+      </c>
+      <c r="B34" t="s">
         <v>98</v>
-      </c>
-      <c r="H33" t="s">
-        <v>99</v>
-      </c>
-    </row>
-    <row r="34" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A34" t="s">
-        <v>0</v>
-      </c>
-      <c r="B34" t="s">
-        <v>100</v>
       </c>
       <c r="C34">
         <v>1020</v>
       </c>
       <c r="D34" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="E34" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="F34">
         <v>6010013110</v>
       </c>
       <c r="G34" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="H34" t="s">
-        <v>104</v>
-      </c>
-    </row>
-    <row r="35" spans="1:8" x14ac:dyDescent="0.2">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="35" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
       <c r="A35" t="s">
         <v>0</v>
       </c>
       <c r="B35" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="C35">
         <v>2110</v>
       </c>
       <c r="D35" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="E35" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="F35">
         <v>6010013020</v>
       </c>
       <c r="G35" t="s">
+        <v>105</v>
+      </c>
+      <c r="H35" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="36" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A36" t="s">
+        <v>0</v>
+      </c>
+      <c r="B36" t="s">
         <v>107</v>
-      </c>
-      <c r="H35" t="s">
-        <v>108</v>
-      </c>
-    </row>
-    <row r="36" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A36" t="s">
-        <v>0</v>
-      </c>
-      <c r="B36" t="s">
-        <v>109</v>
       </c>
       <c r="C36">
         <v>1030</v>
       </c>
       <c r="E36" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="F36">
         <v>35020013035</v>
       </c>
       <c r="G36" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="H36" t="s">
-        <v>112</v>
-      </c>
-    </row>
-    <row r="37" spans="1:8" x14ac:dyDescent="0.2">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="37" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
       <c r="A37" t="s">
         <v>0</v>
       </c>
       <c r="B37" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="C37">
         <v>1400</v>
       </c>
       <c r="E37" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="F37">
         <v>35020013032</v>
       </c>
       <c r="G37" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="H37" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="38" spans="1:8" x14ac:dyDescent="0.2">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="38" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
       <c r="A38" t="s">
         <v>0</v>
       </c>
       <c r="B38" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="C38">
         <v>1410</v>
       </c>
       <c r="E38" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="F38">
         <v>35020013040</v>
       </c>
       <c r="G38" t="s">
+        <v>115</v>
+      </c>
+      <c r="H38" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="39" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A39" t="s">
+        <v>0</v>
+      </c>
+      <c r="B39" t="s">
         <v>117</v>
-      </c>
-      <c r="H38" t="s">
-        <v>118</v>
-      </c>
-    </row>
-    <row r="39" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A39" t="s">
-        <v>0</v>
-      </c>
-      <c r="B39" t="s">
-        <v>119</v>
       </c>
       <c r="C39">
         <v>1010</v>
@@ -3018,53 +3021,53 @@
         <v>6</v>
       </c>
       <c r="E39" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="F39">
         <v>2020013020</v>
       </c>
       <c r="G39" t="s">
+        <v>119</v>
+      </c>
+      <c r="H39" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="40" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A40" t="s">
+        <v>0</v>
+      </c>
+      <c r="B40" t="s">
         <v>121</v>
-      </c>
-      <c r="H39" t="s">
-        <v>122</v>
-      </c>
-    </row>
-    <row r="40" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A40" t="s">
-        <v>0</v>
-      </c>
-      <c r="B40" t="s">
-        <v>123</v>
       </c>
       <c r="C40">
         <v>1100</v>
       </c>
       <c r="E40" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="F40">
         <v>40100013046</v>
       </c>
       <c r="G40" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
       <c r="H40" t="s">
-        <v>126</v>
-      </c>
-    </row>
-    <row r="41" spans="1:8" x14ac:dyDescent="0.2">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="41" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
       <c r="A41" t="s">
         <v>0</v>
       </c>
       <c r="B41" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="C41">
         <v>1200</v>
       </c>
       <c r="E41" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="F41">
         <v>2010013045</v>
@@ -3073,418 +3076,430 @@
         <v>11</v>
       </c>
       <c r="H41" t="s">
-        <v>128</v>
-      </c>
-    </row>
-    <row r="42" spans="1:8" x14ac:dyDescent="0.2">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="42" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
       <c r="A42" t="s">
         <v>0</v>
       </c>
       <c r="B42" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="C42">
         <v>1300</v>
       </c>
       <c r="E42" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="F42">
         <v>40100013042</v>
       </c>
       <c r="G42" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="H42" t="s">
-        <v>131</v>
-      </c>
-    </row>
-    <row r="43" spans="1:8" x14ac:dyDescent="0.2">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="43" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
       <c r="A43" t="s">
         <v>0</v>
       </c>
       <c r="B43" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="C43">
         <v>1610</v>
       </c>
       <c r="E43" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="F43">
         <v>40100013048</v>
       </c>
       <c r="G43" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="H43" t="s">
-        <v>134</v>
-      </c>
-    </row>
-    <row r="44" spans="1:8" x14ac:dyDescent="0.2">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="44" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
       <c r="A44" t="s">
         <v>0</v>
       </c>
       <c r="B44" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="C44">
         <v>2100</v>
       </c>
       <c r="E44" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="F44">
         <v>40130013020</v>
       </c>
       <c r="G44" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="H44" t="s">
-        <v>137</v>
-      </c>
-    </row>
-    <row r="45" spans="1:8" x14ac:dyDescent="0.2">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="45" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
       <c r="A45" t="s">
         <v>0</v>
       </c>
       <c r="B45" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="C45">
         <v>2200</v>
       </c>
       <c r="E45" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
       <c r="F45">
         <v>40130013012</v>
       </c>
       <c r="G45" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="H45" t="s">
-        <v>140</v>
-      </c>
-    </row>
-    <row r="46" spans="1:8" x14ac:dyDescent="0.2">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="46" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
       <c r="A46" t="s">
         <v>0</v>
       </c>
       <c r="B46" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="C46">
         <v>2300</v>
       </c>
       <c r="E46" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="F46">
         <v>40130013020</v>
       </c>
       <c r="G46" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="H46" t="s">
-        <v>142</v>
-      </c>
-    </row>
-    <row r="47" spans="1:8" x14ac:dyDescent="0.2">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="47" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
       <c r="A47" t="s">
         <v>0</v>
       </c>
       <c r="B47" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="C47">
         <v>2710</v>
       </c>
       <c r="E47" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="F47">
         <v>35020013009</v>
       </c>
       <c r="G47" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="H47" t="s">
-        <v>145</v>
-      </c>
-    </row>
-    <row r="48" spans="1:8" x14ac:dyDescent="0.2">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="48" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
       <c r="A48" t="s">
         <v>0</v>
       </c>
       <c r="B48" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="C48">
         <v>2780</v>
       </c>
       <c r="E48" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
       <c r="F48">
         <v>2010013061</v>
       </c>
       <c r="G48" t="s">
+        <v>145</v>
+      </c>
+      <c r="H48" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="49" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A49" t="s">
+        <v>0</v>
+      </c>
+      <c r="B49" t="s">
         <v>147</v>
-      </c>
-      <c r="H48" t="s">
-        <v>148</v>
-      </c>
-    </row>
-    <row r="49" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A49" t="s">
-        <v>0</v>
-      </c>
-      <c r="B49" t="s">
-        <v>149</v>
       </c>
       <c r="C49">
         <v>1010</v>
       </c>
       <c r="D49" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="E49" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="F49">
         <v>32020013200</v>
       </c>
       <c r="G49" t="s">
+        <v>149</v>
+      </c>
+      <c r="H49" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="50" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A50" t="s">
+        <v>0</v>
+      </c>
+      <c r="B50" t="s">
         <v>151</v>
-      </c>
-      <c r="H49" t="s">
-        <v>152</v>
-      </c>
-    </row>
-    <row r="50" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A50" t="s">
-        <v>0</v>
-      </c>
-      <c r="B50" t="s">
-        <v>153</v>
       </c>
       <c r="C50">
         <v>1010</v>
       </c>
       <c r="E50" t="s">
-        <v>154</v>
+        <v>152</v>
       </c>
       <c r="F50">
         <v>39020013003</v>
       </c>
       <c r="G50" t="s">
-        <v>155</v>
+        <v>153</v>
       </c>
       <c r="H50" t="s">
-        <v>156</v>
-      </c>
-    </row>
-    <row r="51" spans="1:8" x14ac:dyDescent="0.2">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="51" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
       <c r="A51" t="s">
         <v>0</v>
       </c>
       <c r="B51" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
       <c r="C51">
         <v>2500</v>
       </c>
       <c r="E51" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
       <c r="F51">
         <v>39020013002</v>
       </c>
       <c r="G51" t="s">
+        <v>156</v>
+      </c>
+      <c r="H51" t="s">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="52" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A52" t="s">
+        <v>0</v>
+      </c>
+      <c r="B52" t="s">
         <v>158</v>
       </c>
-      <c r="H51" t="s">
+      <c r="C52">
+        <v>1010</v>
+      </c>
+      <c r="D52" t="s">
         <v>159</v>
       </c>
-    </row>
-    <row r="52" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A52" t="s">
-        <v>0</v>
-      </c>
-      <c r="B52" t="s">
+      <c r="E52" t="s">
         <v>160</v>
       </c>
-      <c r="C52">
-        <v>1110</v>
-      </c>
-      <c r="E52" t="s">
+      <c r="F52">
+        <v>6020013070</v>
+      </c>
+      <c r="G52" t="s">
         <v>161</v>
       </c>
-      <c r="F52">
-        <v>36010013030</v>
-      </c>
-      <c r="G52" t="s">
+      <c r="H52" t="s">
         <v>162</v>
       </c>
-      <c r="H52" t="s">
+    </row>
+    <row r="53" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A53" t="s">
+        <v>0</v>
+      </c>
+      <c r="B53" t="s">
+        <v>158</v>
+      </c>
+      <c r="C53">
+        <v>2010</v>
+      </c>
+      <c r="D53" t="s">
+        <v>159</v>
+      </c>
+      <c r="E53" t="s">
         <v>163</v>
       </c>
-    </row>
-    <row r="53" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A53" t="s">
-        <v>0</v>
-      </c>
-      <c r="B53" t="s">
-        <v>160</v>
-      </c>
-      <c r="C53">
-        <v>1120</v>
-      </c>
-      <c r="E53" t="s">
+      <c r="F53">
+        <v>6010013116</v>
+      </c>
+      <c r="G53" t="s">
         <v>164</v>
-      </c>
-      <c r="F53">
-        <v>36010013030</v>
-      </c>
-      <c r="G53" t="s">
-        <v>162</v>
       </c>
       <c r="H53" t="s">
         <v>165</v>
       </c>
     </row>
-    <row r="54" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="54" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
       <c r="A54" t="s">
         <v>0</v>
       </c>
       <c r="B54" t="s">
-        <v>160</v>
+        <v>158</v>
       </c>
       <c r="C54">
-        <v>1140</v>
+        <v>2200</v>
+      </c>
+      <c r="D54" t="s">
+        <v>99</v>
       </c>
       <c r="E54" t="s">
         <v>166</v>
       </c>
       <c r="F54">
-        <v>36010013030</v>
+        <v>6010013075</v>
       </c>
       <c r="G54" t="s">
-        <v>162</v>
+        <v>167</v>
       </c>
       <c r="H54" t="s">
-        <v>167</v>
-      </c>
-    </row>
-    <row r="55" spans="1:8" x14ac:dyDescent="0.2">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="55" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
       <c r="A55" t="s">
         <v>0</v>
       </c>
       <c r="B55" t="s">
-        <v>160</v>
+        <v>169</v>
       </c>
       <c r="C55">
-        <v>1145</v>
+        <v>1010</v>
+      </c>
+      <c r="D55" t="s">
+        <v>52</v>
       </c>
       <c r="E55" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
       <c r="F55">
-        <v>36010013030</v>
+        <v>8040013020</v>
       </c>
       <c r="G55" t="s">
-        <v>162</v>
+        <v>171</v>
       </c>
       <c r="H55" t="s">
-        <v>169</v>
-      </c>
-    </row>
-    <row r="56" spans="1:8" x14ac:dyDescent="0.2">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="56" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
       <c r="A56" t="s">
         <v>0</v>
       </c>
       <c r="B56" t="s">
-        <v>170</v>
+        <v>173</v>
       </c>
       <c r="C56">
-        <v>1010</v>
+        <v>1750</v>
       </c>
       <c r="D56" t="s">
-        <v>171</v>
+        <v>103</v>
       </c>
       <c r="E56" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="F56">
-        <v>6020013070</v>
+        <v>1000013100</v>
       </c>
       <c r="G56" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="H56" t="s">
-        <v>174</v>
-      </c>
-    </row>
-    <row r="57" spans="1:8" x14ac:dyDescent="0.2">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="57" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
       <c r="A57" t="s">
         <v>0</v>
       </c>
       <c r="B57" t="s">
-        <v>170</v>
+        <v>177</v>
       </c>
       <c r="C57">
-        <v>2010</v>
+        <v>1020</v>
       </c>
       <c r="D57" t="s">
-        <v>171</v>
+        <v>31</v>
       </c>
       <c r="E57" t="s">
-        <v>175</v>
+        <v>178</v>
       </c>
       <c r="F57">
-        <v>6010013116</v>
+        <v>34010013185</v>
       </c>
       <c r="G57" t="s">
-        <v>176</v>
+        <v>179</v>
       </c>
       <c r="H57" t="s">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="58" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A58" t="s">
+        <v>0</v>
+      </c>
+      <c r="B58" t="s">
         <v>177</v>
       </c>
-    </row>
-    <row r="58" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A58" t="s">
-        <v>0</v>
-      </c>
-      <c r="B58" t="s">
-        <v>170</v>
-      </c>
       <c r="C58">
-        <v>2200</v>
+        <v>1500</v>
       </c>
       <c r="D58" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="E58" t="s">
-        <v>178</v>
+        <v>181</v>
       </c>
       <c r="F58">
-        <v>6010013075</v>
+        <v>34010013197</v>
       </c>
       <c r="G58" t="s">
-        <v>179</v>
+        <v>182</v>
       </c>
       <c r="H58" t="s">
-        <v>180</v>
-      </c>
-    </row>
-    <row r="59" spans="1:8" x14ac:dyDescent="0.2">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="59" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
       <c r="A59" t="s">
         <v>0</v>
       </c>
       <c r="B59" t="s">
-        <v>181</v>
+        <v>184</v>
       </c>
       <c r="C59">
         <v>1010</v>
@@ -3493,114 +3508,111 @@
         <v>52</v>
       </c>
       <c r="E59" t="s">
-        <v>182</v>
+        <v>185</v>
       </c>
       <c r="F59">
-        <v>8040013020</v>
+        <v>8040013030</v>
       </c>
       <c r="G59" t="s">
-        <v>183</v>
+        <v>186</v>
       </c>
       <c r="H59" t="s">
+        <v>187</v>
+      </c>
+    </row>
+    <row r="60" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A60" t="s">
+        <v>0</v>
+      </c>
+      <c r="B60" t="s">
         <v>184</v>
       </c>
-    </row>
-    <row r="60" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A60" t="s">
-        <v>0</v>
-      </c>
-      <c r="B60" t="s">
-        <v>185</v>
-      </c>
       <c r="C60">
-        <v>1750</v>
-      </c>
-      <c r="D60" t="s">
-        <v>105</v>
+        <v>1015</v>
       </c>
       <c r="E60" t="s">
+        <v>188</v>
+      </c>
+      <c r="F60">
+        <v>8040013030</v>
+      </c>
+      <c r="G60" t="s">
         <v>186</v>
       </c>
-      <c r="F60">
-        <v>1000013100</v>
-      </c>
-      <c r="G60" t="s">
-        <v>187</v>
-      </c>
       <c r="H60" t="s">
-        <v>188</v>
-      </c>
-    </row>
-    <row r="61" spans="1:8" x14ac:dyDescent="0.2">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="61" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
       <c r="A61" t="s">
         <v>0</v>
       </c>
       <c r="B61" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="C61">
-        <v>1020</v>
+        <v>1500</v>
       </c>
       <c r="D61" t="s">
-        <v>31</v>
+        <v>103</v>
       </c>
       <c r="E61" t="s">
+        <v>191</v>
+      </c>
+      <c r="F61">
+        <v>9050013090</v>
+      </c>
+      <c r="G61" t="s">
+        <v>192</v>
+      </c>
+      <c r="H61" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="62" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A62" t="s">
+        <v>0</v>
+      </c>
+      <c r="B62" t="s">
         <v>190</v>
       </c>
-      <c r="F61">
-        <v>34010013185</v>
-      </c>
-      <c r="G61" t="s">
-        <v>191</v>
-      </c>
-      <c r="H61" t="s">
+      <c r="C62">
+        <v>1510</v>
+      </c>
+      <c r="D62" t="s">
+        <v>103</v>
+      </c>
+      <c r="E62" t="s">
+        <v>194</v>
+      </c>
+      <c r="F62">
+        <v>9050013090</v>
+      </c>
+      <c r="G62" t="s">
         <v>192</v>
-      </c>
-    </row>
-    <row r="62" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A62" t="s">
-        <v>0</v>
-      </c>
-      <c r="B62" t="s">
-        <v>189</v>
-      </c>
-      <c r="C62">
-        <v>1500</v>
-      </c>
-      <c r="D62" t="s">
-        <v>105</v>
-      </c>
-      <c r="E62" t="s">
-        <v>193</v>
-      </c>
-      <c r="F62">
-        <v>34010013197</v>
-      </c>
-      <c r="G62" t="s">
-        <v>194</v>
       </c>
       <c r="H62" t="s">
         <v>195</v>
       </c>
     </row>
-    <row r="63" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="63" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
       <c r="A63" t="s">
         <v>0</v>
       </c>
       <c r="B63" t="s">
+        <v>190</v>
+      </c>
+      <c r="C63">
+        <v>1700</v>
+      </c>
+      <c r="D63" t="s">
         <v>196</v>
-      </c>
-      <c r="C63">
-        <v>1010</v>
-      </c>
-      <c r="D63" t="s">
-        <v>52</v>
       </c>
       <c r="E63" t="s">
         <v>197</v>
       </c>
       <c r="F63">
-        <v>8040013030</v>
+        <v>9090013010</v>
       </c>
       <c r="G63" t="s">
         <v>198</v>
@@ -3609,278 +3621,269 @@
         <v>199</v>
       </c>
     </row>
-    <row r="64" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="64" spans="1:8" ht="409.6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A64" t="s">
         <v>0</v>
       </c>
       <c r="B64" t="s">
+        <v>190</v>
+      </c>
+      <c r="C64">
+        <v>1700</v>
+      </c>
+      <c r="D64" t="s">
         <v>196</v>
-      </c>
-      <c r="C64">
-        <v>1015</v>
-      </c>
-      <c r="D64" t="s">
-        <v>59</v>
       </c>
       <c r="E64" t="s">
         <v>200</v>
       </c>
       <c r="F64">
-        <v>8040013030</v>
+        <v>9050013050</v>
       </c>
       <c r="G64" t="s">
-        <v>198</v>
-      </c>
-      <c r="H64" t="s">
         <v>201</v>
       </c>
-    </row>
-    <row r="65" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="H64" s="1" t="s">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="65" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
       <c r="A65" t="s">
         <v>0</v>
       </c>
       <c r="B65" t="s">
-        <v>202</v>
+        <v>190</v>
       </c>
       <c r="C65">
-        <v>1500</v>
+        <v>2700</v>
       </c>
       <c r="D65" t="s">
-        <v>105</v>
+        <v>196</v>
       </c>
       <c r="E65" t="s">
         <v>203</v>
       </c>
       <c r="F65">
-        <v>9050013090</v>
+        <v>9090013010</v>
       </c>
       <c r="G65" t="s">
+        <v>198</v>
+      </c>
+      <c r="H65" t="s">
         <v>204</v>
       </c>
-      <c r="H65" t="s">
+    </row>
+    <row r="66" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A66" t="s">
+        <v>0</v>
+      </c>
+      <c r="B66" t="s">
+        <v>190</v>
+      </c>
+      <c r="C66">
+        <v>2700</v>
+      </c>
+      <c r="D66" t="s">
+        <v>103</v>
+      </c>
+      <c r="E66" t="s">
+        <v>203</v>
+      </c>
+      <c r="F66">
+        <v>9090013010</v>
+      </c>
+      <c r="G66" t="s">
+        <v>198</v>
+      </c>
+      <c r="H66" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="67" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A67" t="s">
+        <v>0</v>
+      </c>
+      <c r="B67" t="s">
+        <v>190</v>
+      </c>
+      <c r="C67">
+        <v>2710</v>
+      </c>
+      <c r="D67" t="s">
+        <v>103</v>
+      </c>
+      <c r="E67" t="s">
         <v>205</v>
       </c>
-    </row>
-    <row r="66" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A66" t="s">
-        <v>0</v>
-      </c>
-      <c r="B66" t="s">
-        <v>202</v>
-      </c>
-      <c r="C66">
-        <v>1510</v>
-      </c>
-      <c r="D66" t="s">
-        <v>105</v>
-      </c>
-      <c r="E66" t="s">
+      <c r="F67">
+        <v>9050013050</v>
+      </c>
+      <c r="G67" t="s">
+        <v>201</v>
+      </c>
+      <c r="H67" t="s">
         <v>206</v>
       </c>
-      <c r="F66">
-        <v>9050013090</v>
-      </c>
-      <c r="G66" t="s">
-        <v>204</v>
-      </c>
-      <c r="H66" t="s">
+    </row>
+    <row r="68" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A68" t="s">
+        <v>0</v>
+      </c>
+      <c r="B68" t="s">
+        <v>190</v>
+      </c>
+      <c r="C68">
+        <v>2710</v>
+      </c>
+      <c r="D68" t="s">
+        <v>196</v>
+      </c>
+      <c r="E68" t="s">
+        <v>205</v>
+      </c>
+      <c r="F68">
+        <v>9050013050</v>
+      </c>
+      <c r="G68" t="s">
+        <v>201</v>
+      </c>
+      <c r="H68" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="69" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A69" t="s">
+        <v>0</v>
+      </c>
+      <c r="B69" t="s">
         <v>207</v>
       </c>
-    </row>
-    <row r="67" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A67" t="s">
-        <v>0</v>
-      </c>
-      <c r="B67" t="s">
-        <v>202</v>
-      </c>
-      <c r="C67">
-        <v>1700</v>
-      </c>
-      <c r="D67" t="s">
+      <c r="C69">
+        <v>1000</v>
+      </c>
+      <c r="E69" t="s">
         <v>208</v>
       </c>
-      <c r="E67" t="s">
+      <c r="F69">
+        <v>36010013175</v>
+      </c>
+      <c r="G69" t="s">
         <v>209</v>
       </c>
-      <c r="F67">
-        <v>9090013010</v>
-      </c>
-      <c r="G67" t="s">
+      <c r="H69" t="s">
         <v>210</v>
       </c>
-      <c r="H67" t="s">
+    </row>
+    <row r="70" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A70" t="s">
+        <v>0</v>
+      </c>
+      <c r="B70" t="s">
         <v>211</v>
       </c>
-    </row>
-    <row r="68" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A68" t="s">
-        <v>0</v>
-      </c>
-      <c r="B68" t="s">
-        <v>202</v>
-      </c>
-      <c r="C68">
-        <v>2700</v>
-      </c>
-      <c r="D68" t="s">
-        <v>208</v>
-      </c>
-      <c r="E68" t="s">
+      <c r="C70">
+        <v>1010</v>
+      </c>
+      <c r="E70" t="s">
         <v>212</v>
       </c>
-      <c r="F68">
-        <v>9090013010</v>
-      </c>
-      <c r="G68" t="s">
-        <v>210</v>
-      </c>
-      <c r="H68" t="s">
+      <c r="F70">
+        <v>37010013100</v>
+      </c>
+      <c r="G70" t="s">
         <v>213</v>
       </c>
-    </row>
-    <row r="69" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A69" t="s">
-        <v>0</v>
-      </c>
-      <c r="B69" t="s">
-        <v>202</v>
-      </c>
-      <c r="C69">
-        <v>2700</v>
-      </c>
-      <c r="D69" t="s">
-        <v>105</v>
-      </c>
-      <c r="E69" t="s">
-        <v>212</v>
-      </c>
-      <c r="F69">
-        <v>9090013010</v>
-      </c>
-      <c r="G69" t="s">
-        <v>210</v>
-      </c>
-      <c r="H69" t="s">
-        <v>213</v>
-      </c>
-    </row>
-    <row r="70" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A70" t="s">
-        <v>0</v>
-      </c>
-      <c r="B70" t="s">
-        <v>202</v>
-      </c>
-      <c r="C70">
-        <v>2710</v>
-      </c>
-      <c r="D70" t="s">
-        <v>208</v>
-      </c>
-      <c r="E70" t="s">
+      <c r="H70" t="s">
         <v>214</v>
       </c>
-      <c r="F70">
-        <v>9050013050</v>
-      </c>
-      <c r="G70" t="s">
+    </row>
+    <row r="71" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A71" t="s">
+        <v>0</v>
+      </c>
+      <c r="B71" t="s">
         <v>215</v>
       </c>
-      <c r="H70" t="s">
+      <c r="C71">
+        <v>1010</v>
+      </c>
+      <c r="D71" t="s">
+        <v>99</v>
+      </c>
+      <c r="E71" t="s">
         <v>216</v>
       </c>
-    </row>
-    <row r="71" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A71" t="s">
-        <v>0</v>
-      </c>
-      <c r="B71" t="s">
-        <v>202</v>
-      </c>
-      <c r="C71">
-        <v>2710</v>
-      </c>
-      <c r="D71" t="s">
-        <v>105</v>
-      </c>
-      <c r="E71" t="s">
-        <v>214</v>
-      </c>
       <c r="F71">
-        <v>9050013050</v>
+        <v>6010013080</v>
       </c>
       <c r="G71" t="s">
-        <v>215</v>
+        <v>217</v>
       </c>
       <c r="H71" t="s">
-        <v>216</v>
-      </c>
-    </row>
-    <row r="72" spans="1:8" x14ac:dyDescent="0.2">
+        <v>218</v>
+      </c>
+    </row>
+    <row r="72" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
       <c r="A72" t="s">
         <v>0</v>
       </c>
       <c r="B72" t="s">
-        <v>217</v>
+        <v>219</v>
       </c>
       <c r="C72">
-        <v>1000</v>
+        <v>1100</v>
       </c>
       <c r="E72" t="s">
-        <v>218</v>
+        <v>220</v>
       </c>
       <c r="F72">
-        <v>36010013175</v>
+        <v>35010013025</v>
       </c>
       <c r="G72" t="s">
+        <v>221</v>
+      </c>
+      <c r="H72" t="s">
+        <v>222</v>
+      </c>
+    </row>
+    <row r="73" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A73" t="s">
+        <v>0</v>
+      </c>
+      <c r="B73" t="s">
         <v>219</v>
       </c>
-      <c r="H72" t="s">
-        <v>220</v>
-      </c>
-    </row>
-    <row r="73" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A73" t="s">
-        <v>0</v>
-      </c>
-      <c r="B73" t="s">
-        <v>221</v>
-      </c>
       <c r="C73">
-        <v>1010</v>
+        <v>1200</v>
       </c>
       <c r="E73" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="F73">
-        <v>37010013100</v>
+        <v>35010013041</v>
       </c>
       <c r="G73" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="H73" t="s">
-        <v>224</v>
-      </c>
-    </row>
-    <row r="74" spans="1:8" x14ac:dyDescent="0.2">
+        <v>225</v>
+      </c>
+    </row>
+    <row r="74" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
       <c r="A74" t="s">
         <v>0</v>
       </c>
       <c r="B74" t="s">
-        <v>225</v>
+        <v>219</v>
       </c>
       <c r="C74">
-        <v>1010</v>
-      </c>
-      <c r="D74" t="s">
-        <v>101</v>
+        <v>1500</v>
       </c>
       <c r="E74" t="s">
         <v>226</v>
       </c>
       <c r="F74">
-        <v>6010013080</v>
+        <v>35020013042</v>
       </c>
       <c r="G74" t="s">
         <v>227</v>
@@ -3889,67 +3892,67 @@
         <v>228</v>
       </c>
     </row>
-    <row r="75" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="75" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
       <c r="A75" t="s">
         <v>0</v>
       </c>
       <c r="B75" t="s">
+        <v>219</v>
+      </c>
+      <c r="C75">
+        <v>2400</v>
+      </c>
+      <c r="E75" t="s">
         <v>229</v>
       </c>
-      <c r="C75">
-        <v>1100</v>
-      </c>
-      <c r="E75" t="s">
+      <c r="F75">
+        <v>35010013030</v>
+      </c>
+      <c r="G75" t="s">
         <v>230</v>
       </c>
-      <c r="F75">
-        <v>35010013025</v>
-      </c>
-      <c r="G75" t="s">
+      <c r="H75" t="s">
         <v>231</v>
       </c>
-      <c r="H75" t="s">
+    </row>
+    <row r="76" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A76" t="s">
+        <v>0</v>
+      </c>
+      <c r="B76" t="s">
+        <v>219</v>
+      </c>
+      <c r="C76">
+        <v>2700</v>
+      </c>
+      <c r="E76" t="s">
         <v>232</v>
       </c>
-    </row>
-    <row r="76" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A76" t="s">
-        <v>0</v>
-      </c>
-      <c r="B76" t="s">
-        <v>229</v>
-      </c>
-      <c r="C76">
+      <c r="F76">
+        <v>35010013036</v>
+      </c>
+      <c r="G76" t="s">
+        <v>233</v>
+      </c>
+      <c r="H76" t="s">
+        <v>234</v>
+      </c>
+    </row>
+    <row r="77" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A77" t="s">
+        <v>0</v>
+      </c>
+      <c r="B77" t="s">
+        <v>235</v>
+      </c>
+      <c r="C77">
         <v>1200</v>
-      </c>
-      <c r="E76" t="s">
-        <v>233</v>
-      </c>
-      <c r="F76">
-        <v>35010013041</v>
-      </c>
-      <c r="G76" t="s">
-        <v>234</v>
-      </c>
-      <c r="H76" t="s">
-        <v>235</v>
-      </c>
-    </row>
-    <row r="77" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A77" t="s">
-        <v>0</v>
-      </c>
-      <c r="B77" t="s">
-        <v>229</v>
-      </c>
-      <c r="C77">
-        <v>1500</v>
       </c>
       <c r="E77" t="s">
         <v>236</v>
       </c>
       <c r="F77">
-        <v>35020013042</v>
+        <v>35020013012</v>
       </c>
       <c r="G77" t="s">
         <v>237</v>
@@ -3958,21 +3961,21 @@
         <v>238</v>
       </c>
     </row>
-    <row r="78" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="78" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
       <c r="A78" t="s">
         <v>0</v>
       </c>
       <c r="B78" t="s">
-        <v>229</v>
+        <v>235</v>
       </c>
       <c r="C78">
-        <v>2400</v>
+        <v>1300</v>
       </c>
       <c r="E78" t="s">
         <v>239</v>
       </c>
       <c r="F78">
-        <v>35010013030</v>
+        <v>35020013060</v>
       </c>
       <c r="G78" t="s">
         <v>240</v>
@@ -3981,44 +3984,44 @@
         <v>241</v>
       </c>
     </row>
-    <row r="79" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="79" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
       <c r="A79" t="s">
         <v>0</v>
       </c>
       <c r="B79" t="s">
+        <v>235</v>
+      </c>
+      <c r="C79">
+        <v>2000</v>
+      </c>
+      <c r="E79" t="s">
         <v>242</v>
       </c>
-      <c r="C79">
-        <v>1200</v>
-      </c>
-      <c r="E79" t="s">
+      <c r="F79">
+        <v>35020013007</v>
+      </c>
+      <c r="G79" t="s">
         <v>243</v>
       </c>
-      <c r="F79">
-        <v>35020013012</v>
-      </c>
-      <c r="G79" t="s">
+      <c r="H79" t="s">
         <v>244</v>
       </c>
-      <c r="H79" t="s">
+    </row>
+    <row r="80" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A80" t="s">
+        <v>0</v>
+      </c>
+      <c r="B80" t="s">
         <v>245</v>
       </c>
-    </row>
-    <row r="80" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A80" t="s">
-        <v>0</v>
-      </c>
-      <c r="B80" t="s">
-        <v>242</v>
-      </c>
       <c r="C80">
-        <v>1300</v>
+        <v>1010</v>
       </c>
       <c r="E80" t="s">
         <v>246</v>
       </c>
       <c r="F80">
-        <v>35020013060</v>
+        <v>7070013060</v>
       </c>
       <c r="G80" t="s">
         <v>247</v>
@@ -4027,44 +4030,50 @@
         <v>248</v>
       </c>
     </row>
-    <row r="81" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="81" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
       <c r="A81" t="s">
         <v>0</v>
       </c>
       <c r="B81" t="s">
-        <v>242</v>
+        <v>245</v>
       </c>
       <c r="C81">
-        <v>2000</v>
+        <v>1030</v>
+      </c>
+      <c r="D81" t="s">
+        <v>249</v>
       </c>
       <c r="E81" t="s">
+        <v>250</v>
+      </c>
+      <c r="F81">
+        <v>7070013090</v>
+      </c>
+      <c r="G81" t="s">
+        <v>251</v>
+      </c>
+      <c r="H81" t="s">
+        <v>252</v>
+      </c>
+    </row>
+    <row r="82" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A82" t="s">
+        <v>0</v>
+      </c>
+      <c r="B82" t="s">
+        <v>245</v>
+      </c>
+      <c r="C82">
+        <v>1040</v>
+      </c>
+      <c r="D82" t="s">
         <v>249</v>
-      </c>
-      <c r="F81">
-        <v>35020013007</v>
-      </c>
-      <c r="G81" t="s">
-        <v>250</v>
-      </c>
-      <c r="H81" t="s">
-        <v>251</v>
-      </c>
-    </row>
-    <row r="82" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A82" t="s">
-        <v>0</v>
-      </c>
-      <c r="B82" t="s">
-        <v>252</v>
-      </c>
-      <c r="C82">
-        <v>1010</v>
       </c>
       <c r="E82" t="s">
         <v>253</v>
       </c>
       <c r="F82">
-        <v>7070013060</v>
+        <v>7060013010</v>
       </c>
       <c r="G82" t="s">
         <v>254</v>
@@ -4073,330 +4082,324 @@
         <v>255</v>
       </c>
     </row>
-    <row r="83" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="83" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
       <c r="A83" t="s">
         <v>0</v>
       </c>
       <c r="B83" t="s">
-        <v>252</v>
+        <v>245</v>
       </c>
       <c r="C83">
-        <v>1030</v>
+        <v>1050</v>
       </c>
       <c r="D83" t="s">
+        <v>249</v>
+      </c>
+      <c r="E83" t="s">
         <v>256</v>
       </c>
-      <c r="E83" t="s">
+      <c r="F83">
+        <v>7040013020</v>
+      </c>
+      <c r="G83" t="s">
         <v>257</v>
       </c>
-      <c r="F83">
-        <v>7070013090</v>
-      </c>
-      <c r="G83" t="s">
+      <c r="H83" t="s">
         <v>258</v>
       </c>
-      <c r="H83" t="s">
+    </row>
+    <row r="84" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A84" t="s">
+        <v>0</v>
+      </c>
+      <c r="B84" t="s">
+        <v>245</v>
+      </c>
+      <c r="C84">
+        <v>1060</v>
+      </c>
+      <c r="D84" t="s">
+        <v>249</v>
+      </c>
+      <c r="E84" t="s">
         <v>259</v>
       </c>
-    </row>
-    <row r="84" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A84" t="s">
-        <v>0</v>
-      </c>
-      <c r="B84" t="s">
-        <v>252</v>
-      </c>
-      <c r="C84">
-        <v>1040</v>
-      </c>
-      <c r="D84" t="s">
-        <v>256</v>
-      </c>
-      <c r="E84" t="s">
+      <c r="F84">
+        <v>7070013010</v>
+      </c>
+      <c r="G84" t="s">
         <v>260</v>
       </c>
-      <c r="F84">
-        <v>7060013010</v>
-      </c>
-      <c r="G84" t="s">
+      <c r="H84" t="s">
         <v>261</v>
       </c>
-      <c r="H84" t="s">
+    </row>
+    <row r="85" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A85" t="s">
+        <v>0</v>
+      </c>
+      <c r="B85" t="s">
+        <v>245</v>
+      </c>
+      <c r="C85">
+        <v>1080</v>
+      </c>
+      <c r="D85" t="s">
+        <v>249</v>
+      </c>
+      <c r="E85" t="s">
         <v>262</v>
-      </c>
-    </row>
-    <row r="85" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A85" t="s">
-        <v>0</v>
-      </c>
-      <c r="B85" t="s">
-        <v>252</v>
-      </c>
-      <c r="C85">
-        <v>1050</v>
-      </c>
-      <c r="D85" t="s">
-        <v>256</v>
-      </c>
-      <c r="E85" t="s">
-        <v>263</v>
       </c>
       <c r="F85">
         <v>7040013020</v>
       </c>
       <c r="G85" t="s">
+        <v>257</v>
+      </c>
+      <c r="H85" t="s">
+        <v>263</v>
+      </c>
+    </row>
+    <row r="86" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A86" t="s">
+        <v>0</v>
+      </c>
+      <c r="B86" t="s">
+        <v>245</v>
+      </c>
+      <c r="C86">
+        <v>1100</v>
+      </c>
+      <c r="E86" t="s">
         <v>264</v>
       </c>
-      <c r="H85" t="s">
+      <c r="F86">
+        <v>7040013010</v>
+      </c>
+      <c r="G86" t="s">
         <v>265</v>
       </c>
-    </row>
-    <row r="86" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A86" t="s">
-        <v>0</v>
-      </c>
-      <c r="B86" t="s">
-        <v>252</v>
-      </c>
-      <c r="C86">
-        <v>1060</v>
-      </c>
-      <c r="D86" t="s">
-        <v>256</v>
-      </c>
-      <c r="E86" t="s">
+      <c r="H86" t="s">
         <v>266</v>
       </c>
-      <c r="F86">
-        <v>7070013010</v>
-      </c>
-      <c r="G86" t="s">
+    </row>
+    <row r="87" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A87" t="s">
+        <v>0</v>
+      </c>
+      <c r="B87" t="s">
+        <v>245</v>
+      </c>
+      <c r="C87">
+        <v>1210</v>
+      </c>
+      <c r="D87" t="s">
+        <v>249</v>
+      </c>
+      <c r="E87" t="s">
         <v>267</v>
       </c>
-      <c r="H86" t="s">
+      <c r="F87">
+        <v>7040013010</v>
+      </c>
+      <c r="G87" t="s">
+        <v>265</v>
+      </c>
+      <c r="H87" t="s">
         <v>268</v>
       </c>
     </row>
-    <row r="87" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A87" t="s">
-        <v>0</v>
-      </c>
-      <c r="B87" t="s">
-        <v>252</v>
-      </c>
-      <c r="C87">
-        <v>1080</v>
-      </c>
-      <c r="D87" t="s">
-        <v>256</v>
-      </c>
-      <c r="E87" t="s">
+    <row r="88" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A88" t="s">
+        <v>0</v>
+      </c>
+      <c r="B88" t="s">
+        <v>245</v>
+      </c>
+      <c r="C88">
+        <v>1220</v>
+      </c>
+      <c r="D88" t="s">
+        <v>249</v>
+      </c>
+      <c r="E88" t="s">
         <v>269</v>
-      </c>
-      <c r="F87">
-        <v>7040013020</v>
-      </c>
-      <c r="G87" t="s">
-        <v>264</v>
-      </c>
-      <c r="H87" t="s">
-        <v>270</v>
-      </c>
-    </row>
-    <row r="88" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A88" t="s">
-        <v>0</v>
-      </c>
-      <c r="B88" t="s">
-        <v>252</v>
-      </c>
-      <c r="C88">
-        <v>1100</v>
-      </c>
-      <c r="E88" t="s">
-        <v>271</v>
       </c>
       <c r="F88">
         <v>7040013010</v>
       </c>
       <c r="G88" t="s">
-        <v>272</v>
+        <v>265</v>
       </c>
       <c r="H88" t="s">
-        <v>273</v>
-      </c>
-    </row>
-    <row r="89" spans="1:8" x14ac:dyDescent="0.2">
+        <v>270</v>
+      </c>
+    </row>
+    <row r="89" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
       <c r="A89" t="s">
         <v>0</v>
       </c>
       <c r="B89" t="s">
-        <v>252</v>
+        <v>245</v>
       </c>
       <c r="C89">
-        <v>1210</v>
+        <v>2210</v>
       </c>
       <c r="D89" t="s">
-        <v>256</v>
+        <v>249</v>
       </c>
       <c r="E89" t="s">
-        <v>274</v>
+        <v>271</v>
       </c>
       <c r="F89">
         <v>7040013010</v>
       </c>
       <c r="G89" t="s">
+        <v>265</v>
+      </c>
+      <c r="H89" t="s">
         <v>272</v>
       </c>
-      <c r="H89" t="s">
+    </row>
+    <row r="90" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A90" t="s">
+        <v>0</v>
+      </c>
+      <c r="B90" t="s">
+        <v>273</v>
+      </c>
+      <c r="C90">
+        <v>1000</v>
+      </c>
+      <c r="E90" t="s">
+        <v>274</v>
+      </c>
+      <c r="F90">
+        <v>38010013052</v>
+      </c>
+      <c r="G90" t="s">
         <v>275</v>
       </c>
-    </row>
-    <row r="90" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A90" t="s">
-        <v>0</v>
-      </c>
-      <c r="B90" t="s">
-        <v>252</v>
-      </c>
-      <c r="C90">
-        <v>1220</v>
-      </c>
-      <c r="D90" t="s">
-        <v>256</v>
-      </c>
-      <c r="E90" t="s">
+      <c r="H90" t="s">
         <v>276</v>
       </c>
-      <c r="F90">
-        <v>7040013010</v>
-      </c>
-      <c r="G90" t="s">
-        <v>272</v>
-      </c>
-      <c r="H90" t="s">
+    </row>
+    <row r="91" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A91" t="s">
+        <v>0</v>
+      </c>
+      <c r="B91" t="s">
+        <v>273</v>
+      </c>
+      <c r="C91">
+        <v>1005</v>
+      </c>
+      <c r="E91" t="s">
         <v>277</v>
       </c>
-    </row>
-    <row r="91" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A91" t="s">
-        <v>0</v>
-      </c>
-      <c r="B91" t="s">
-        <v>252</v>
-      </c>
-      <c r="C91">
-        <v>2210</v>
-      </c>
-      <c r="D91" t="s">
-        <v>256</v>
-      </c>
-      <c r="E91" t="s">
+      <c r="F91">
+        <v>38010013052</v>
+      </c>
+      <c r="G91" t="s">
+        <v>275</v>
+      </c>
+      <c r="H91" t="s">
         <v>278</v>
       </c>
-      <c r="F91">
-        <v>7040013010</v>
-      </c>
-      <c r="G91" t="s">
-        <v>272</v>
-      </c>
-      <c r="H91" t="s">
+    </row>
+    <row r="92" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A92" t="s">
+        <v>0</v>
+      </c>
+      <c r="B92" t="s">
+        <v>273</v>
+      </c>
+      <c r="C92">
+        <v>1100</v>
+      </c>
+      <c r="E92" t="s">
         <v>279</v>
       </c>
-    </row>
-    <row r="92" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A92" t="s">
-        <v>0</v>
-      </c>
-      <c r="B92" t="s">
+      <c r="F92">
+        <v>38010013011</v>
+      </c>
+      <c r="G92" t="s">
         <v>280</v>
       </c>
-      <c r="C92">
-        <v>1380</v>
-      </c>
-      <c r="E92" t="s">
+      <c r="H92" t="s">
         <v>281</v>
       </c>
-      <c r="F92">
-        <v>40010013010</v>
-      </c>
-      <c r="G92" t="s">
+    </row>
+    <row r="93" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A93" t="s">
+        <v>0</v>
+      </c>
+      <c r="B93" t="s">
         <v>282</v>
       </c>
-      <c r="H92" t="s">
+      <c r="C93">
+        <v>2600</v>
+      </c>
+      <c r="E93" t="s">
         <v>283</v>
       </c>
-    </row>
-    <row r="93" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A93" t="s">
-        <v>0</v>
-      </c>
-      <c r="B93" t="s">
-        <v>280</v>
-      </c>
-      <c r="C93">
-        <v>1385</v>
-      </c>
-      <c r="E93" t="s">
+      <c r="F93">
+        <v>32020013220</v>
+      </c>
+      <c r="G93" t="s">
         <v>284</v>
-      </c>
-      <c r="F93">
-        <v>40010013010</v>
-      </c>
-      <c r="G93" t="s">
-        <v>282</v>
       </c>
       <c r="H93" t="s">
         <v>285</v>
       </c>
     </row>
-    <row r="94" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="94" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
       <c r="A94" t="s">
         <v>0</v>
       </c>
       <c r="B94" t="s">
+        <v>282</v>
+      </c>
+      <c r="C94">
+        <v>2640</v>
+      </c>
+      <c r="E94" t="s">
         <v>286</v>
       </c>
-      <c r="C94">
-        <v>1000</v>
-      </c>
-      <c r="E94" t="s">
+      <c r="F94">
+        <v>32020013140</v>
+      </c>
+      <c r="G94" t="s">
         <v>287</v>
       </c>
-      <c r="F94">
-        <v>38010013052</v>
-      </c>
-      <c r="G94" t="s">
+      <c r="H94" t="s">
         <v>288</v>
       </c>
-      <c r="H94" t="s">
+    </row>
+    <row r="95" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A95" t="s">
+        <v>0</v>
+      </c>
+      <c r="B95" t="s">
+        <v>282</v>
+      </c>
+      <c r="C95" t="s">
         <v>289</v>
-      </c>
-    </row>
-    <row r="95" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A95" t="s">
-        <v>0</v>
-      </c>
-      <c r="B95" t="s">
-        <v>286</v>
-      </c>
-      <c r="C95">
-        <v>1005</v>
       </c>
       <c r="E95" t="s">
         <v>290</v>
       </c>
       <c r="F95">
-        <v>38010013052</v>
+        <v>32020013220</v>
       </c>
       <c r="G95" t="s">
-        <v>288</v>
+        <v>284</v>
       </c>
       <c r="H95" t="s">
         <v>291</v>
       </c>
     </row>
-    <row r="96" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="96" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
       <c r="A96" t="s">
         <v>0</v>
       </c>
@@ -4404,13 +4407,16 @@
         <v>292</v>
       </c>
       <c r="C96">
-        <v>2600</v>
+        <v>1010</v>
+      </c>
+      <c r="D96" t="s">
+        <v>6</v>
       </c>
       <c r="E96" t="s">
         <v>293</v>
       </c>
       <c r="F96">
-        <v>32020013220</v>
+        <v>2040013020</v>
       </c>
       <c r="G96" t="s">
         <v>294</v>
@@ -4419,53 +4425,53 @@
         <v>295</v>
       </c>
     </row>
-    <row r="97" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="97" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
       <c r="A97" t="s">
         <v>0</v>
       </c>
       <c r="B97" t="s">
-        <v>292</v>
+        <v>296</v>
       </c>
       <c r="C97">
-        <v>2640</v>
+        <v>1005</v>
       </c>
       <c r="E97" t="s">
+        <v>297</v>
+      </c>
+      <c r="F97">
+        <v>36010013190</v>
+      </c>
+      <c r="G97" t="s">
+        <v>298</v>
+      </c>
+      <c r="H97" t="s">
+        <v>299</v>
+      </c>
+    </row>
+    <row r="98" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A98" t="s">
+        <v>0</v>
+      </c>
+      <c r="B98" t="s">
         <v>296</v>
       </c>
-      <c r="F97">
-        <v>32020013140</v>
-      </c>
-      <c r="G97" t="s">
-        <v>297</v>
-      </c>
-      <c r="H97" t="s">
-        <v>298</v>
-      </c>
-    </row>
-    <row r="98" spans="1:8" ht="409.6" x14ac:dyDescent="0.2">
-      <c r="A98" t="s">
-        <v>0</v>
-      </c>
-      <c r="B98" t="s">
-        <v>292</v>
-      </c>
-      <c r="C98" t="s">
-        <v>299</v>
+      <c r="C98">
+        <v>1007</v>
       </c>
       <c r="E98" t="s">
         <v>300</v>
       </c>
       <c r="F98">
-        <v>32020013220</v>
+        <v>36010013190</v>
       </c>
       <c r="G98" t="s">
-        <v>294</v>
-      </c>
-      <c r="H98" s="1" t="s">
+        <v>298</v>
+      </c>
+      <c r="H98" t="s">
         <v>301</v>
       </c>
     </row>
-    <row r="99" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="99" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
       <c r="A99" t="s">
         <v>0</v>
       </c>
@@ -4473,16 +4479,16 @@
         <v>302</v>
       </c>
       <c r="C99">
-        <v>1010</v>
+        <v>2050</v>
       </c>
       <c r="D99" t="s">
-        <v>6</v>
+        <v>99</v>
       </c>
       <c r="E99" t="s">
         <v>303</v>
       </c>
       <c r="F99">
-        <v>2040013020</v>
+        <v>9090013902</v>
       </c>
       <c r="G99" t="s">
         <v>304</v>
@@ -4491,7 +4497,7 @@
         <v>305</v>
       </c>
     </row>
-    <row r="100" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="100" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
       <c r="A100" t="s">
         <v>0</v>
       </c>
@@ -4499,13 +4505,16 @@
         <v>306</v>
       </c>
       <c r="C100">
-        <v>1005</v>
+        <v>1010</v>
+      </c>
+      <c r="D100" t="s">
+        <v>52</v>
       </c>
       <c r="E100" t="s">
         <v>307</v>
       </c>
       <c r="F100">
-        <v>36010013190</v>
+        <v>8060013020</v>
       </c>
       <c r="G100" t="s">
         <v>308</v>
@@ -4514,7 +4523,7 @@
         <v>309</v>
       </c>
     </row>
-    <row r="101" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="101" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
       <c r="A101" t="s">
         <v>0</v>
       </c>
@@ -4522,13 +4531,13 @@
         <v>306</v>
       </c>
       <c r="C101">
-        <v>1007</v>
+        <v>1015</v>
       </c>
       <c r="E101" t="s">
         <v>310</v>
       </c>
       <c r="F101">
-        <v>36010013190</v>
+        <v>8060013020</v>
       </c>
       <c r="G101" t="s">
         <v>308</v>
@@ -4537,206 +4546,194 @@
         <v>311</v>
       </c>
     </row>
-    <row r="102" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="102" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
       <c r="A102" t="s">
         <v>0</v>
       </c>
       <c r="B102" t="s">
+        <v>306</v>
+      </c>
+      <c r="C102">
+        <v>1040</v>
+      </c>
+      <c r="D102" t="s">
+        <v>52</v>
+      </c>
+      <c r="E102" t="s">
         <v>312</v>
       </c>
-      <c r="C102">
-        <v>2050</v>
-      </c>
-      <c r="D102" t="s">
-        <v>101</v>
-      </c>
-      <c r="E102" t="s">
+      <c r="F102">
+        <v>8060013010</v>
+      </c>
+      <c r="G102" t="s">
         <v>313</v>
       </c>
-      <c r="F102">
-        <v>9090013902</v>
-      </c>
-      <c r="G102" t="s">
+      <c r="H102" t="s">
         <v>314</v>
       </c>
-      <c r="H102" t="s">
+    </row>
+    <row r="103" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A103" t="s">
+        <v>0</v>
+      </c>
+      <c r="B103" t="s">
+        <v>306</v>
+      </c>
+      <c r="C103">
+        <v>1045</v>
+      </c>
+      <c r="E103" t="s">
         <v>315</v>
       </c>
-    </row>
-    <row r="103" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A103" t="s">
-        <v>0</v>
-      </c>
-      <c r="B103" t="s">
+      <c r="F103">
+        <v>8060013010</v>
+      </c>
+      <c r="G103" t="s">
+        <v>313</v>
+      </c>
+      <c r="H103" t="s">
         <v>316</v>
       </c>
-      <c r="C103">
-        <v>1010</v>
-      </c>
-      <c r="D103" t="s">
+    </row>
+    <row r="104" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A104" t="s">
+        <v>0</v>
+      </c>
+      <c r="B104" t="s">
+        <v>306</v>
+      </c>
+      <c r="C104">
+        <v>2010</v>
+      </c>
+      <c r="D104" t="s">
         <v>52</v>
       </c>
-      <c r="E103" t="s">
+      <c r="E104" t="s">
         <v>317</v>
-      </c>
-      <c r="F103">
-        <v>8060013020</v>
-      </c>
-      <c r="G103" t="s">
-        <v>318</v>
-      </c>
-      <c r="H103" t="s">
-        <v>319</v>
-      </c>
-    </row>
-    <row r="104" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A104" t="s">
-        <v>0</v>
-      </c>
-      <c r="B104" t="s">
-        <v>316</v>
-      </c>
-      <c r="C104">
-        <v>1015</v>
-      </c>
-      <c r="D104" t="s">
-        <v>59</v>
-      </c>
-      <c r="E104" t="s">
-        <v>320</v>
       </c>
       <c r="F104">
         <v>8060013020</v>
       </c>
       <c r="G104" t="s">
+        <v>308</v>
+      </c>
+      <c r="H104" t="s">
         <v>318</v>
       </c>
-      <c r="H104" t="s">
+    </row>
+    <row r="105" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A105" t="s">
+        <v>0</v>
+      </c>
+      <c r="B105" t="s">
+        <v>306</v>
+      </c>
+      <c r="C105">
+        <v>2015</v>
+      </c>
+      <c r="D105" t="s">
+        <v>63</v>
+      </c>
+      <c r="E105" t="s">
+        <v>319</v>
+      </c>
+      <c r="F105">
+        <v>8060013020</v>
+      </c>
+      <c r="G105" t="s">
+        <v>308</v>
+      </c>
+      <c r="H105" t="s">
+        <v>320</v>
+      </c>
+    </row>
+    <row r="106" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A106" t="s">
+        <v>0</v>
+      </c>
+      <c r="B106" t="s">
         <v>321</v>
       </c>
-    </row>
-    <row r="105" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A105" t="s">
-        <v>0</v>
-      </c>
-      <c r="B105" t="s">
-        <v>316</v>
-      </c>
-      <c r="C105">
-        <v>1040</v>
-      </c>
-      <c r="D105" t="s">
-        <v>52</v>
-      </c>
-      <c r="E105" t="s">
+      <c r="C106">
+        <v>1100</v>
+      </c>
+      <c r="D106" t="s">
+        <v>196</v>
+      </c>
+      <c r="E106" t="s">
         <v>322</v>
       </c>
-      <c r="F105">
-        <v>8060013010</v>
-      </c>
-      <c r="G105" t="s">
-        <v>323</v>
-      </c>
-      <c r="H105" t="s">
-        <v>324</v>
-      </c>
-    </row>
-    <row r="106" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A106" t="s">
-        <v>0</v>
-      </c>
-      <c r="B106" t="s">
-        <v>316</v>
-      </c>
-      <c r="C106">
-        <v>1045</v>
-      </c>
-      <c r="D106" t="s">
-        <v>59</v>
-      </c>
-      <c r="E106" t="s">
-        <v>325</v>
-      </c>
       <c r="F106">
-        <v>8060013010</v>
+        <v>9060013020</v>
       </c>
       <c r="G106" t="s">
         <v>323</v>
       </c>
       <c r="H106" t="s">
+        <v>324</v>
+      </c>
+    </row>
+    <row r="107" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A107" t="s">
+        <v>0</v>
+      </c>
+      <c r="B107" t="s">
+        <v>325</v>
+      </c>
+      <c r="C107">
+        <v>3116</v>
+      </c>
+      <c r="E107" t="s">
         <v>326</v>
       </c>
-    </row>
-    <row r="107" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A107" t="s">
-        <v>0</v>
-      </c>
-      <c r="B107" t="s">
-        <v>316</v>
-      </c>
-      <c r="C107">
-        <v>2010</v>
-      </c>
-      <c r="D107" t="s">
-        <v>52</v>
-      </c>
-      <c r="E107" t="s">
+      <c r="F107">
+        <v>3250013065</v>
+      </c>
+      <c r="G107" t="s">
         <v>327</v>
-      </c>
-      <c r="F107">
-        <v>8060013020</v>
-      </c>
-      <c r="G107" t="s">
-        <v>318</v>
       </c>
       <c r="H107" t="s">
         <v>328</v>
       </c>
     </row>
-    <row r="108" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="108" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
       <c r="A108" t="s">
         <v>0</v>
       </c>
       <c r="B108" t="s">
-        <v>316</v>
+        <v>325</v>
       </c>
       <c r="C108">
-        <v>2015</v>
-      </c>
-      <c r="D108" t="s">
-        <v>59</v>
+        <v>3117</v>
       </c>
       <c r="E108" t="s">
         <v>329</v>
       </c>
       <c r="F108">
-        <v>8060013020</v>
+        <v>3250013066</v>
       </c>
       <c r="G108" t="s">
-        <v>318</v>
+        <v>330</v>
       </c>
       <c r="H108" t="s">
-        <v>330</v>
-      </c>
-    </row>
-    <row r="109" spans="1:8" x14ac:dyDescent="0.2">
+        <v>331</v>
+      </c>
+    </row>
+    <row r="109" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
       <c r="A109" t="s">
         <v>0</v>
       </c>
       <c r="B109" t="s">
-        <v>331</v>
+        <v>325</v>
       </c>
       <c r="C109">
-        <v>1100</v>
-      </c>
-      <c r="D109" t="s">
-        <v>208</v>
+        <v>3118</v>
       </c>
       <c r="E109" t="s">
         <v>332</v>
       </c>
       <c r="F109">
-        <v>9060013020</v>
+        <v>3250013067</v>
       </c>
       <c r="G109" t="s">
         <v>333</v>
@@ -4745,7 +4742,7 @@
         <v>334</v>
       </c>
     </row>
-    <row r="110" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="110" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
       <c r="A110" t="s">
         <v>0</v>
       </c>
@@ -4756,7 +4753,7 @@
         <v>1010</v>
       </c>
       <c r="D110" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="E110" t="s">
         <v>336</v>
@@ -4771,7 +4768,7 @@
         <v>338</v>
       </c>
     </row>
-    <row r="111" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="111" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
       <c r="A111" t="s">
         <v>0</v>
       </c>
@@ -4782,7 +4779,7 @@
         <v>1100</v>
       </c>
       <c r="D111" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="E111" t="s">
         <v>339</v>
@@ -4791,13 +4788,13 @@
         <v>34010013197</v>
       </c>
       <c r="G111" t="s">
-        <v>194</v>
+        <v>182</v>
       </c>
       <c r="H111" t="s">
         <v>340</v>
       </c>
     </row>
-    <row r="112" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="112" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
       <c r="A112" t="s">
         <v>0</v>
       </c>
@@ -4820,7 +4817,7 @@
         <v>344</v>
       </c>
     </row>
-    <row r="113" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="113" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
       <c r="A113" t="s">
         <v>0</v>
       </c>
@@ -4831,7 +4828,7 @@
         <v>1010</v>
       </c>
       <c r="D113" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="E113" t="s">
         <v>346</v>
@@ -4846,7 +4843,7 @@
         <v>348</v>
       </c>
     </row>
-    <row r="114" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="114" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
       <c r="A114" t="s">
         <v>0</v>
       </c>
@@ -4872,7 +4869,7 @@
         <v>352</v>
       </c>
     </row>
-    <row r="115" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="115" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
       <c r="A115" t="s">
         <v>0</v>
       </c>
@@ -4898,7 +4895,7 @@
         <v>355</v>
       </c>
     </row>
-    <row r="116" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="116" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
       <c r="A116" t="s">
         <v>0</v>
       </c>
@@ -4924,7 +4921,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="117" spans="1:8" ht="409.6" x14ac:dyDescent="0.2">
+    <row r="117" spans="1:8" ht="409.6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A117" t="s">
         <v>0</v>
       </c>
@@ -4950,7 +4947,7 @@
         <v>360</v>
       </c>
     </row>
-    <row r="118" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="118" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
       <c r="A118" t="s">
         <v>0</v>
       </c>
@@ -4960,9 +4957,6 @@
       <c r="C118">
         <v>3116</v>
       </c>
-      <c r="D118" t="s">
-        <v>17</v>
-      </c>
       <c r="E118" t="s">
         <v>361</v>
       </c>
@@ -4976,7 +4970,7 @@
         <v>363</v>
       </c>
     </row>
-    <row r="119" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="119" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
       <c r="A119" t="s">
         <v>0</v>
       </c>
@@ -4986,9 +4980,6 @@
       <c r="C119">
         <v>3117</v>
       </c>
-      <c r="D119" t="s">
-        <v>17</v>
-      </c>
       <c r="E119" t="s">
         <v>364</v>
       </c>
@@ -5002,7 +4993,7 @@
         <v>366</v>
       </c>
     </row>
-    <row r="120" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="120" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
       <c r="A120" t="s">
         <v>0</v>
       </c>
@@ -5012,9 +5003,6 @@
       <c r="C120">
         <v>3118</v>
       </c>
-      <c r="D120" t="s">
-        <v>17</v>
-      </c>
       <c r="E120" t="s">
         <v>367</v>
       </c>
@@ -5028,7 +5016,7 @@
         <v>369</v>
       </c>
     </row>
-    <row r="121" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="121" spans="1:8" hidden="1" x14ac:dyDescent="0.2">
       <c r="A121" t="s">
         <v>0</v>
       </c>
@@ -5055,6 +5043,13 @@
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="A1:H121" xr:uid="{F61A08E9-A0F5-9448-A2BC-A228F6060EDB}">
+    <filterColumn colId="1">
+      <filters>
+        <filter val="CHEM"/>
+      </filters>
+    </filterColumn>
+  </autoFilter>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>